<commit_message>
update generate paths with selected branches
</commit_message>
<xml_diff>
--- a/ScratchData/data.xlsx
+++ b/ScratchData/data.xlsx
@@ -1,14 +1,15 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <fileVersion appName="xl" lastEdited="5" lowestEdited="5" rupBuild="27729"/>
+  <fileVersion appName="xl" lastEdited="5" lowestEdited="5" rupBuild="28028"/>
   <workbookPr showInkAnnotation="0" autoCompressPictures="0"/>
   <bookViews>
-    <workbookView xWindow="5080" yWindow="8200" windowWidth="27380" windowHeight="20100" tabRatio="500" activeTab="1"/>
+    <workbookView xWindow="-20" yWindow="0" windowWidth="30520" windowHeight="16020" tabRatio="500" activeTab="2"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
     <sheet name="time" sheetId="2" r:id="rId2"/>
+    <sheet name="Sheet2" sheetId="3" r:id="rId3"/>
   </sheets>
   <calcPr calcId="140000" concurrentCalc="0"/>
   <extLst>
@@ -20,7 +21,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="749" uniqueCount="270">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="775" uniqueCount="294">
   <si>
     <t>Done in 748</t>
   </si>
@@ -830,6 +831,78 @@
   </si>
   <si>
     <t>D = 9 pred</t>
+  </si>
+  <si>
+    <t>BaloonFactory</t>
+  </si>
+  <si>
+    <t>Class</t>
+  </si>
+  <si>
+    <t>Method name</t>
+  </si>
+  <si>
+    <t>Method id</t>
+  </si>
+  <si>
+    <t>getLines</t>
+  </si>
+  <si>
+    <t>Path</t>
+  </si>
+  <si>
+    <t>Full time</t>
+  </si>
+  <si>
+    <t>getTextBounds</t>
+  </si>
+  <si>
+    <t>max</t>
+  </si>
+  <si>
+    <t>min</t>
+  </si>
+  <si>
+    <t>unsats</t>
+  </si>
+  <si>
+    <t>addPadding</t>
+  </si>
+  <si>
+    <t>no branches</t>
+  </si>
+  <si>
+    <t>correctHorizontaly</t>
+  </si>
+  <si>
+    <t>no good branches</t>
+  </si>
+  <si>
+    <t>correctVericaly</t>
+  </si>
+  <si>
+    <t>isInsideBounds</t>
+  </si>
+  <si>
+    <t>without loop</t>
+  </si>
+  <si>
+    <t>run time without loops</t>
+  </si>
+  <si>
+    <t>7000?</t>
+  </si>
+  <si>
+    <t>getCirlcePath</t>
+  </si>
+  <si>
+    <t>less</t>
+  </si>
+  <si>
+    <t>0 unsats without loops</t>
+  </si>
+  <si>
+    <t>getNormalPath</t>
   </si>
 </sst>
 </file>
@@ -4775,4 +4848,202 @@
     </ext>
   </extLst>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+  <dimension ref="A1:J9"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0"/>
+  <cols>
+    <col min="2" max="2" width="12.83203125" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:10">
+      <c r="A1" t="s">
+        <v>271</v>
+      </c>
+      <c r="B1" t="s">
+        <v>272</v>
+      </c>
+      <c r="C1" t="s">
+        <v>273</v>
+      </c>
+      <c r="D1" t="s">
+        <v>275</v>
+      </c>
+      <c r="E1" t="s">
+        <v>276</v>
+      </c>
+      <c r="F1" t="s">
+        <v>278</v>
+      </c>
+      <c r="G1" t="s">
+        <v>279</v>
+      </c>
+      <c r="H1" t="s">
+        <v>280</v>
+      </c>
+      <c r="I1" t="s">
+        <v>287</v>
+      </c>
+      <c r="J1" t="s">
+        <v>288</v>
+      </c>
+    </row>
+    <row r="2" spans="1:10">
+      <c r="A2" t="s">
+        <v>270</v>
+      </c>
+      <c r="B2" t="s">
+        <v>274</v>
+      </c>
+      <c r="C2">
+        <v>1</v>
+      </c>
+      <c r="D2">
+        <v>16</v>
+      </c>
+      <c r="E2">
+        <v>7590</v>
+      </c>
+      <c r="F2">
+        <v>4698</v>
+      </c>
+      <c r="G2">
+        <v>1295</v>
+      </c>
+      <c r="H2">
+        <v>11</v>
+      </c>
+      <c r="I2">
+        <v>0</v>
+      </c>
+      <c r="J2" t="s">
+        <v>289</v>
+      </c>
+    </row>
+    <row r="3" spans="1:10">
+      <c r="B3" t="s">
+        <v>277</v>
+      </c>
+      <c r="C3">
+        <v>2</v>
+      </c>
+      <c r="D3">
+        <v>15</v>
+      </c>
+      <c r="E3">
+        <v>1029</v>
+      </c>
+      <c r="F3">
+        <v>986</v>
+      </c>
+      <c r="G3">
+        <v>338</v>
+      </c>
+      <c r="H3">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="4" spans="1:10">
+      <c r="B4" t="s">
+        <v>281</v>
+      </c>
+      <c r="C4">
+        <v>3</v>
+      </c>
+      <c r="D4" t="s">
+        <v>282</v>
+      </c>
+    </row>
+    <row r="5" spans="1:10">
+      <c r="B5" t="s">
+        <v>283</v>
+      </c>
+      <c r="C5">
+        <v>4</v>
+      </c>
+      <c r="D5" t="s">
+        <v>284</v>
+      </c>
+    </row>
+    <row r="6" spans="1:10">
+      <c r="B6" t="s">
+        <v>285</v>
+      </c>
+      <c r="C6">
+        <v>5</v>
+      </c>
+      <c r="D6" t="s">
+        <v>284</v>
+      </c>
+    </row>
+    <row r="7" spans="1:10">
+      <c r="B7" t="s">
+        <v>286</v>
+      </c>
+      <c r="C7">
+        <v>6</v>
+      </c>
+      <c r="D7">
+        <v>5</v>
+      </c>
+      <c r="E7">
+        <v>752</v>
+      </c>
+      <c r="F7">
+        <v>700</v>
+      </c>
+      <c r="G7">
+        <v>91</v>
+      </c>
+      <c r="H7">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="8" spans="1:10">
+      <c r="B8" t="s">
+        <v>290</v>
+      </c>
+      <c r="C8">
+        <v>7</v>
+      </c>
+      <c r="D8">
+        <v>20736</v>
+      </c>
+      <c r="E8">
+        <v>4486</v>
+      </c>
+      <c r="F8">
+        <v>4300</v>
+      </c>
+      <c r="G8">
+        <v>4100</v>
+      </c>
+      <c r="I8" t="s">
+        <v>291</v>
+      </c>
+      <c r="J8" t="s">
+        <v>292</v>
+      </c>
+    </row>
+    <row r="9" spans="1:10">
+      <c r="B9" t="s">
+        <v>293</v>
+      </c>
+      <c r="C9">
+        <v>8</v>
+      </c>
+      <c r="D9" t="s">
+        <v>282</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <extLst>
+    <ext xmlns:mx="http://schemas.microsoft.com/office/mac/excel/2008/main" uri="{64002731-A6B0-56B0-2670-7721B7C09600}">
+      <mx:PLV Mode="0" OnePage="0" WScale="0"/>
+    </ext>
+  </extLst>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
fixed some bugs, so can run on Base64 methods
</commit_message>
<xml_diff>
--- a/ScratchData/data.xlsx
+++ b/ScratchData/data.xlsx
@@ -4,12 +4,13 @@
   <fileVersion appName="xl" lastEdited="5" lowestEdited="5" rupBuild="28028"/>
   <workbookPr showInkAnnotation="0" autoCompressPictures="0"/>
   <bookViews>
-    <workbookView xWindow="-20" yWindow="0" windowWidth="30520" windowHeight="16020" tabRatio="500" activeTab="2"/>
+    <workbookView xWindow="-20" yWindow="0" windowWidth="31020" windowHeight="16020" tabRatio="500" activeTab="2"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
     <sheet name="time" sheetId="2" r:id="rId2"/>
     <sheet name="Sheet2" sheetId="3" r:id="rId3"/>
+    <sheet name="Sheet3" sheetId="4" r:id="rId4"/>
   </sheets>
   <calcPr calcId="140000" concurrentCalc="0"/>
   <extLst>
@@ -21,7 +22,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="775" uniqueCount="294">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="801" uniqueCount="318">
   <si>
     <t>Done in 748</t>
   </si>
@@ -899,10 +900,82 @@
     <t>less</t>
   </si>
   <si>
+    <t>0 unsats</t>
+  </si>
+  <si>
     <t>0 unsats without loops</t>
   </si>
   <si>
     <t>getNormalPath</t>
+  </si>
+  <si>
+    <t>getArrow</t>
+  </si>
+  <si>
+    <t>1f,2t,3f</t>
+  </si>
+  <si>
+    <t>1f,2f</t>
+  </si>
+  <si>
+    <t>1t,5t,7f,8t,9t,10t,11t</t>
+  </si>
+  <si>
+    <t>1t,5f,6f</t>
+  </si>
+  <si>
+    <t>1t,5t,7f,8t,9t,10t,11f</t>
+  </si>
+  <si>
+    <t>1f,2t,3t,4f</t>
+  </si>
+  <si>
+    <t>1t,5t,7t</t>
+  </si>
+  <si>
+    <t>1t,5t,7f,8f,10t,11f</t>
+  </si>
+  <si>
+    <t>1t,5t,7f,8t,9t,10f</t>
+  </si>
+  <si>
+    <t>1t,5t,7f,8f,10f</t>
+  </si>
+  <si>
+    <t>1t,5t,7f,8t,9f,10t,11f</t>
+  </si>
+  <si>
+    <t>1t,5f,6t</t>
+  </si>
+  <si>
+    <t>1t,5t,7f,8t,9f,10f</t>
+  </si>
+  <si>
+    <t>1t,5t,7f,8f,10t,11t</t>
+  </si>
+  <si>
+    <t>1f,2t,3t,4t</t>
+  </si>
+  <si>
+    <t>1t,5t,7f,8t,9f,10t,11t</t>
+  </si>
+  <si>
+    <t>Base64</t>
+  </si>
+  <si>
+    <t>getBytes</t>
+  </si>
+  <si>
+    <t>encode</t>
+  </si>
+  <si>
+    <t>fillElementWithBigIteger</t>
+  </si>
+  <si>
+    <t>decode</t>
+  </si>
+  <si>
+    <t>isWhite</t>
   </si>
 </sst>
 </file>
@@ -934,12 +1007,18 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="2">
+  <fills count="3">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFFF00"/>
+        <bgColor indexed="64"/>
+      </patternFill>
     </fill>
   </fills>
   <borders count="1">
@@ -990,8 +1069,9 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
   </cellXfs>
   <cellStyles count="37">
     <cellStyle name="Followed Hyperlink" xfId="2" builtinId="9" hidden="1"/>
@@ -4852,7 +4932,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:J9"/>
+  <dimension ref="A1:J15"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0"/>
   <cols>
     <col min="2" max="2" width="12.83203125" bestFit="1" customWidth="1"/>
@@ -5024,18 +5104,111 @@
         <v>291</v>
       </c>
       <c r="J8" t="s">
-        <v>292</v>
+        <v>293</v>
       </c>
     </row>
     <row r="9" spans="1:10">
       <c r="B9" t="s">
-        <v>293</v>
+        <v>294</v>
       </c>
       <c r="C9">
         <v>8</v>
       </c>
       <c r="D9" t="s">
         <v>282</v>
+      </c>
+    </row>
+    <row r="10" spans="1:10">
+      <c r="B10" t="s">
+        <v>295</v>
+      </c>
+      <c r="C10">
+        <v>9</v>
+      </c>
+      <c r="D10">
+        <v>10</v>
+      </c>
+      <c r="E10">
+        <v>1997</v>
+      </c>
+      <c r="F10">
+        <v>700</v>
+      </c>
+      <c r="G10">
+        <v>18</v>
+      </c>
+      <c r="I10" t="s">
+        <v>292</v>
+      </c>
+    </row>
+    <row r="11" spans="1:10">
+      <c r="A11" t="s">
+        <v>312</v>
+      </c>
+      <c r="B11" t="s">
+        <v>313</v>
+      </c>
+      <c r="C11">
+        <v>2</v>
+      </c>
+      <c r="D11">
+        <v>4</v>
+      </c>
+      <c r="E11">
+        <v>1144</v>
+      </c>
+      <c r="F11">
+        <v>1092</v>
+      </c>
+    </row>
+    <row r="12" spans="1:10">
+      <c r="B12" t="s">
+        <v>314</v>
+      </c>
+      <c r="C12">
+        <v>4</v>
+      </c>
+      <c r="D12">
+        <v>4</v>
+      </c>
+      <c r="E12">
+        <v>1151</v>
+      </c>
+      <c r="F12">
+        <v>1090</v>
+      </c>
+    </row>
+    <row r="13" spans="1:10">
+      <c r="B13" t="s">
+        <v>315</v>
+      </c>
+      <c r="C13">
+        <v>7</v>
+      </c>
+      <c r="D13" t="s">
+        <v>284</v>
+      </c>
+    </row>
+    <row r="14" spans="1:10">
+      <c r="B14" t="s">
+        <v>316</v>
+      </c>
+      <c r="C14">
+        <v>8</v>
+      </c>
+      <c r="D14" t="s">
+        <v>284</v>
+      </c>
+    </row>
+    <row r="15" spans="1:10">
+      <c r="B15" t="s">
+        <v>317</v>
+      </c>
+      <c r="C15">
+        <v>13</v>
+      </c>
+      <c r="D15">
+        <v>5</v>
       </c>
     </row>
   </sheetData>
@@ -5046,4 +5219,105 @@
     </ext>
   </extLst>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+  <dimension ref="A1:A16"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0"/>
+  <cols>
+    <col min="1" max="1" width="18" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:1">
+      <c r="A1" t="s">
+        <v>297</v>
+      </c>
+    </row>
+    <row r="2" spans="1:1">
+      <c r="A2" t="s">
+        <v>296</v>
+      </c>
+    </row>
+    <row r="3" spans="1:1">
+      <c r="A3" t="s">
+        <v>301</v>
+      </c>
+    </row>
+    <row r="4" spans="1:1">
+      <c r="A4" t="s">
+        <v>310</v>
+      </c>
+    </row>
+    <row r="5" spans="1:1">
+      <c r="A5" s="1" t="s">
+        <v>299</v>
+      </c>
+    </row>
+    <row r="6" spans="1:1">
+      <c r="A6" s="1" t="s">
+        <v>307</v>
+      </c>
+    </row>
+    <row r="7" spans="1:1">
+      <c r="A7" t="s">
+        <v>305</v>
+      </c>
+    </row>
+    <row r="8" spans="1:1">
+      <c r="A8" t="s">
+        <v>303</v>
+      </c>
+    </row>
+    <row r="9" spans="1:1">
+      <c r="A9" t="s">
+        <v>309</v>
+      </c>
+    </row>
+    <row r="10" spans="1:1">
+      <c r="A10" t="s">
+        <v>308</v>
+      </c>
+    </row>
+    <row r="11" spans="1:1">
+      <c r="A11" t="s">
+        <v>306</v>
+      </c>
+    </row>
+    <row r="12" spans="1:1">
+      <c r="A12" t="s">
+        <v>311</v>
+      </c>
+    </row>
+    <row r="13" spans="1:1">
+      <c r="A13" t="s">
+        <v>304</v>
+      </c>
+    </row>
+    <row r="14" spans="1:1">
+      <c r="A14" t="s">
+        <v>300</v>
+      </c>
+    </row>
+    <row r="15" spans="1:1">
+      <c r="A15" t="s">
+        <v>298</v>
+      </c>
+    </row>
+    <row r="16" spans="1:1">
+      <c r="A16" t="s">
+        <v>302</v>
+      </c>
+    </row>
+  </sheetData>
+  <sortState ref="A1:A16">
+    <sortCondition ref="A1"/>
+  </sortState>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <extLst>
+    <ext xmlns:mx="http://schemas.microsoft.com/office/mac/excel/2008/main" uri="{64002731-A6B0-56B0-2670-7721B7C09600}">
+      <mx:PLV Mode="0" OnePage="0" WScale="0"/>
+    </ext>
+  </extLst>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
code for processing sat/unsat counts and updated excel data
</commit_message>
<xml_diff>
--- a/ScratchData/data.xlsx
+++ b/ScratchData/data.xlsx
@@ -1,10 +1,10 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <fileVersion appName="xl" lastEdited="5" lowestEdited="5" rupBuild="28125"/>
+  <fileVersion appName="xl" lastEdited="5" lowestEdited="5" rupBuild="27729"/>
   <workbookPr showInkAnnotation="0" autoCompressPictures="0"/>
   <bookViews>
-    <workbookView xWindow="4600" yWindow="720" windowWidth="28780" windowHeight="16320" tabRatio="500" activeTab="4"/>
+    <workbookView xWindow="240" yWindow="240" windowWidth="25360" windowHeight="14740" tabRatio="500" activeTab="4"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -1366,9 +1366,6 @@
     <t>Path id</t>
   </si>
   <si>
-    <t xml:space="preserve">Path </t>
-  </si>
-  <si>
     <t>Path time</t>
   </si>
   <si>
@@ -1391,6 +1388,9 @@
   </si>
   <si>
     <t>%</t>
+  </si>
+  <si>
+    <t>Paths</t>
   </si>
 </sst>
 </file>
@@ -1452,8 +1452,10 @@
       <diagonal/>
     </border>
   </borders>
-  <cellStyleXfs count="77">
+  <cellStyleXfs count="79">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
@@ -1539,7 +1541,7 @@
     <xf numFmtId="2" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="2" fontId="0" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1"/>
   </cellXfs>
-  <cellStyles count="77">
+  <cellStyles count="79">
     <cellStyle name="Followed Hyperlink" xfId="2" builtinId="9" hidden="1"/>
     <cellStyle name="Followed Hyperlink" xfId="4" builtinId="9" hidden="1"/>
     <cellStyle name="Followed Hyperlink" xfId="6" builtinId="9" hidden="1"/>
@@ -1578,6 +1580,7 @@
     <cellStyle name="Followed Hyperlink" xfId="72" builtinId="9" hidden="1"/>
     <cellStyle name="Followed Hyperlink" xfId="74" builtinId="9" hidden="1"/>
     <cellStyle name="Followed Hyperlink" xfId="76" builtinId="9" hidden="1"/>
+    <cellStyle name="Followed Hyperlink" xfId="78" builtinId="9" hidden="1"/>
     <cellStyle name="Hyperlink" xfId="1" builtinId="8" hidden="1"/>
     <cellStyle name="Hyperlink" xfId="3" builtinId="8" hidden="1"/>
     <cellStyle name="Hyperlink" xfId="5" builtinId="8" hidden="1"/>
@@ -1616,6 +1619,7 @@
     <cellStyle name="Hyperlink" xfId="71" builtinId="8" hidden="1"/>
     <cellStyle name="Hyperlink" xfId="73" builtinId="8" hidden="1"/>
     <cellStyle name="Hyperlink" xfId="75" builtinId="8" hidden="1"/>
+    <cellStyle name="Hyperlink" xfId="77" builtinId="8" hidden="1"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
@@ -5599,7 +5603,7 @@
         <v>752</v>
       </c>
       <c r="F7" s="4">
-        <f t="shared" ref="F4:F67" si="0">(E7-G7)/E7</f>
+        <f t="shared" ref="F7:F65" si="0">(E7-G7)/E7</f>
         <v>6.9148936170212769E-2</v>
       </c>
       <c r="G7">
@@ -6953,7 +6957,7 @@
         <v>4302</v>
       </c>
       <c r="F69" s="4">
-        <f t="shared" ref="F68:F105" si="1">(E69-G69)/E69</f>
+        <f t="shared" ref="F69:F105" si="1">(E69-G69)/E69</f>
         <v>0.44932589493258951</v>
       </c>
       <c r="G69">
@@ -9901,31 +9905,31 @@
         <v>272</v>
       </c>
       <c r="D1" s="2" t="s">
+        <v>446</v>
+      </c>
+      <c r="E1" s="2" t="s">
+        <v>455</v>
+      </c>
+      <c r="F1" s="2" t="s">
         <v>275</v>
       </c>
-      <c r="E1" s="2" t="s">
-        <v>446</v>
-      </c>
-      <c r="F1" s="2" t="s">
+      <c r="G1" s="2" t="s">
         <v>447</v>
       </c>
-      <c r="G1" s="2" t="s">
-        <v>448</v>
-      </c>
       <c r="H1" s="2" t="s">
-        <v>455</v>
+        <v>454</v>
       </c>
       <c r="I1" s="2" t="s">
-        <v>451</v>
+        <v>450</v>
       </c>
       <c r="J1" s="2" t="s">
         <v>452</v>
       </c>
       <c r="K1" s="2" t="s">
+        <v>451</v>
+      </c>
+      <c r="L1" s="2" t="s">
         <v>453</v>
-      </c>
-      <c r="L1" s="2" t="s">
-        <v>454</v>
       </c>
     </row>
     <row r="2" spans="1:12">
@@ -9938,67 +9942,127 @@
       <c r="C2" s="2">
         <v>1</v>
       </c>
-      <c r="D2" s="2">
+      <c r="D2">
+        <v>1</v>
+      </c>
+      <c r="E2" t="s">
+        <v>210</v>
+      </c>
+      <c r="F2" s="2">
         <f>AVERAGE(7641,7431,7353)</f>
         <v>7475</v>
       </c>
-      <c r="E2">
-        <v>1</v>
-      </c>
-      <c r="F2" t="s">
-        <v>210</v>
-      </c>
       <c r="G2">
         <v>7169</v>
       </c>
       <c r="H2" s="4">
-        <f>G2/$D$2</f>
+        <f>G2/F2</f>
         <v>0.95906354515050163</v>
       </c>
+      <c r="I2">
+        <v>45</v>
+      </c>
+      <c r="J2">
+        <v>0</v>
+      </c>
+      <c r="K2">
+        <v>4</v>
+      </c>
+      <c r="L2">
+        <v>0</v>
+      </c>
     </row>
     <row r="3" spans="1:12">
-      <c r="E3">
+      <c r="D3">
         <v>2</v>
       </c>
-      <c r="F3" t="s">
-        <v>449</v>
+      <c r="E3" t="s">
+        <v>448</v>
+      </c>
+      <c r="F3" s="2">
+        <f t="shared" ref="F3:F5" si="0">AVERAGE(7641,7431,7353)</f>
+        <v>7475</v>
       </c>
       <c r="G3">
         <v>7283</v>
       </c>
       <c r="H3" s="4">
-        <f t="shared" ref="H3:H5" si="0">G3/$D$2</f>
+        <f t="shared" ref="H3:H5" si="1">G3/F3</f>
         <v>0.97431438127090297</v>
       </c>
+      <c r="I3">
+        <v>47</v>
+      </c>
+      <c r="J3">
+        <v>0</v>
+      </c>
+      <c r="K3">
+        <v>2</v>
+      </c>
+      <c r="L3">
+        <v>0</v>
+      </c>
     </row>
     <row r="4" spans="1:12">
-      <c r="E4">
-        <v>3</v>
-      </c>
-      <c r="F4" t="s">
-        <v>450</v>
+      <c r="D4">
+        <v>3</v>
+      </c>
+      <c r="E4" t="s">
+        <v>449</v>
+      </c>
+      <c r="F4" s="2">
+        <f t="shared" si="0"/>
+        <v>7475</v>
       </c>
       <c r="G4">
         <v>7367</v>
       </c>
       <c r="H4" s="4">
+        <f t="shared" si="1"/>
+        <v>0.9855518394648829</v>
+      </c>
+      <c r="I4">
+        <v>49</v>
+      </c>
+      <c r="J4">
+        <v>0</v>
+      </c>
+      <c r="K4">
+        <v>0</v>
+      </c>
+      <c r="L4">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="5" spans="1:12">
+      <c r="D5">
+        <v>4</v>
+      </c>
+      <c r="E5" t="s">
+        <v>211</v>
+      </c>
+      <c r="F5" s="2">
         <f t="shared" si="0"/>
-        <v>0.9855518394648829</v>
-      </c>
-    </row>
-    <row r="5" spans="1:12">
-      <c r="E5">
-        <v>4</v>
-      </c>
-      <c r="F5" t="s">
-        <v>211</v>
+        <v>7475</v>
       </c>
       <c r="G5">
         <v>7902</v>
       </c>
       <c r="H5" s="4">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>1.0571237458193981</v>
+      </c>
+      <c r="I5">
+        <v>49</v>
+      </c>
+      <c r="J5">
+        <v>0</v>
+      </c>
+      <c r="K5">
+        <v>0</v>
+      </c>
+      <c r="L5">
+        <v>0</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
scripts for running the analysis and collecting the data
</commit_message>
<xml_diff>
--- a/ScratchData/data.xlsx
+++ b/ScratchData/data.xlsx
@@ -1,10 +1,10 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <fileVersion appName="xl" lastEdited="5" lowestEdited="5" rupBuild="27729"/>
+  <fileVersion appName="xl" lastEdited="5" lowestEdited="5" rupBuild="28125"/>
   <workbookPr showInkAnnotation="0" autoCompressPictures="0"/>
   <bookViews>
-    <workbookView xWindow="240" yWindow="240" windowWidth="25360" windowHeight="14740" tabRatio="500" activeTab="4"/>
+    <workbookView xWindow="5260" yWindow="0" windowWidth="25440" windowHeight="14740" tabRatio="500" firstSheet="1" activeTab="5"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -12,6 +12,9 @@
     <sheet name="Sheet2" sheetId="3" r:id="rId3"/>
     <sheet name="cleanedData" sheetId="4" r:id="rId4"/>
     <sheet name="TestPathData" sheetId="5" r:id="rId5"/>
+    <sheet name="Time Data" sheetId="6" r:id="rId6"/>
+    <sheet name="SatUnsatData" sheetId="7" r:id="rId7"/>
+    <sheet name="Sheet5" sheetId="8" r:id="rId8"/>
   </sheets>
   <calcPr calcId="140000" concurrentCalc="0"/>
   <extLst>
@@ -23,7 +26,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1199" uniqueCount="456">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1286" uniqueCount="486">
   <si>
     <t>Done in 748</t>
   </si>
@@ -1391,6 +1394,96 @@
   </si>
   <si>
     <t>Paths</t>
+  </si>
+  <si>
+    <t>Path Id</t>
+  </si>
+  <si>
+    <t>Path Time</t>
+  </si>
+  <si>
+    <t>test.BallonFactory</t>
+  </si>
+  <si>
+    <t>1t3f4f</t>
+  </si>
+  <si>
+    <t>1f2t3f4f</t>
+  </si>
+  <si>
+    <t>1t3t5f6f</t>
+  </si>
+  <si>
+    <t>1t3f4t5f6f</t>
+  </si>
+  <si>
+    <t>1f2t3t5f6f</t>
+  </si>
+  <si>
+    <t>1t3t5t</t>
+  </si>
+  <si>
+    <t>1f2t3f4t5f6f</t>
+  </si>
+  <si>
+    <t>1t3t5f6t</t>
+  </si>
+  <si>
+    <t>1t3f4t5t</t>
+  </si>
+  <si>
+    <t>1f2t3t5t</t>
+  </si>
+  <si>
+    <t>1f2t3t5f6t</t>
+  </si>
+  <si>
+    <t>1f2t3f4t5t</t>
+  </si>
+  <si>
+    <t>1t3f4t5f6t</t>
+  </si>
+  <si>
+    <t>1f2t3f4t5f6t</t>
+  </si>
+  <si>
+    <t>1t</t>
+  </si>
+  <si>
+    <t>1f2f3t</t>
+  </si>
+  <si>
+    <t>1f2f3f4f</t>
+  </si>
+  <si>
+    <t>1t5t7t</t>
+  </si>
+  <si>
+    <t>1f2t3t4t</t>
+  </si>
+  <si>
+    <t>1f2t3t4f</t>
+  </si>
+  <si>
+    <t>1f2t3f</t>
+  </si>
+  <si>
+    <t>1t5t7f8f10t</t>
+  </si>
+  <si>
+    <t>1t5f</t>
+  </si>
+  <si>
+    <t>1t5t7f8f10f</t>
+  </si>
+  <si>
+    <t>1t5t7f8t10t</t>
+  </si>
+  <si>
+    <t>1t5t7f8t10f</t>
+  </si>
+  <si>
+    <t>1f2f3f4t</t>
   </si>
 </sst>
 </file>
@@ -1452,8 +1545,16 @@
       <diagonal/>
     </border>
   </borders>
-  <cellStyleXfs count="79">
+  <cellStyleXfs count="87">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
@@ -1541,7 +1642,7 @@
     <xf numFmtId="2" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="2" fontId="0" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1"/>
   </cellXfs>
-  <cellStyles count="79">
+  <cellStyles count="87">
     <cellStyle name="Followed Hyperlink" xfId="2" builtinId="9" hidden="1"/>
     <cellStyle name="Followed Hyperlink" xfId="4" builtinId="9" hidden="1"/>
     <cellStyle name="Followed Hyperlink" xfId="6" builtinId="9" hidden="1"/>
@@ -1581,6 +1682,10 @@
     <cellStyle name="Followed Hyperlink" xfId="74" builtinId="9" hidden="1"/>
     <cellStyle name="Followed Hyperlink" xfId="76" builtinId="9" hidden="1"/>
     <cellStyle name="Followed Hyperlink" xfId="78" builtinId="9" hidden="1"/>
+    <cellStyle name="Followed Hyperlink" xfId="80" builtinId="9" hidden="1"/>
+    <cellStyle name="Followed Hyperlink" xfId="82" builtinId="9" hidden="1"/>
+    <cellStyle name="Followed Hyperlink" xfId="84" builtinId="9" hidden="1"/>
+    <cellStyle name="Followed Hyperlink" xfId="86" builtinId="9" hidden="1"/>
     <cellStyle name="Hyperlink" xfId="1" builtinId="8" hidden="1"/>
     <cellStyle name="Hyperlink" xfId="3" builtinId="8" hidden="1"/>
     <cellStyle name="Hyperlink" xfId="5" builtinId="8" hidden="1"/>
@@ -1620,6 +1725,10 @@
     <cellStyle name="Hyperlink" xfId="73" builtinId="8" hidden="1"/>
     <cellStyle name="Hyperlink" xfId="75" builtinId="8" hidden="1"/>
     <cellStyle name="Hyperlink" xfId="77" builtinId="8" hidden="1"/>
+    <cellStyle name="Hyperlink" xfId="79" builtinId="8" hidden="1"/>
+    <cellStyle name="Hyperlink" xfId="81" builtinId="8" hidden="1"/>
+    <cellStyle name="Hyperlink" xfId="83" builtinId="8" hidden="1"/>
+    <cellStyle name="Hyperlink" xfId="85" builtinId="8" hidden="1"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
@@ -10074,4 +10183,955 @@
     </ext>
   </extLst>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+  <dimension ref="A1:G35"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0"/>
+  <sheetData>
+    <row r="1" spans="1:7">
+      <c r="A1" t="s">
+        <v>270</v>
+      </c>
+      <c r="B1" t="s">
+        <v>272</v>
+      </c>
+      <c r="C1" t="s">
+        <v>274</v>
+      </c>
+      <c r="D1" t="s">
+        <v>456</v>
+      </c>
+      <c r="E1" t="s">
+        <v>275</v>
+      </c>
+      <c r="F1" t="s">
+        <v>457</v>
+      </c>
+      <c r="G1" t="s">
+        <v>454</v>
+      </c>
+    </row>
+    <row r="2" spans="1:7">
+      <c r="A2" t="s">
+        <v>458</v>
+      </c>
+      <c r="B2">
+        <v>1</v>
+      </c>
+      <c r="C2" t="s">
+        <v>210</v>
+      </c>
+      <c r="D2">
+        <v>1</v>
+      </c>
+      <c r="E2">
+        <v>7586</v>
+      </c>
+      <c r="F2">
+        <v>7421</v>
+      </c>
+      <c r="G2" s="4">
+        <f>F2/E2</f>
+        <v>0.97824940680200367</v>
+      </c>
+    </row>
+    <row r="3" spans="1:7">
+      <c r="A3" t="s">
+        <v>458</v>
+      </c>
+      <c r="B3">
+        <v>1</v>
+      </c>
+      <c r="C3" t="s">
+        <v>448</v>
+      </c>
+      <c r="D3">
+        <v>2</v>
+      </c>
+      <c r="E3">
+        <v>7586</v>
+      </c>
+      <c r="F3">
+        <v>7469</v>
+      </c>
+      <c r="G3" s="4">
+        <f t="shared" ref="G3:G35" si="0">F3/E3</f>
+        <v>0.98457685209596624</v>
+      </c>
+    </row>
+    <row r="4" spans="1:7">
+      <c r="A4" t="s">
+        <v>458</v>
+      </c>
+      <c r="B4">
+        <v>1</v>
+      </c>
+      <c r="C4" t="s">
+        <v>449</v>
+      </c>
+      <c r="D4">
+        <v>3</v>
+      </c>
+      <c r="E4">
+        <v>7586</v>
+      </c>
+      <c r="F4">
+        <v>7493</v>
+      </c>
+      <c r="G4" s="4">
+        <f t="shared" si="0"/>
+        <v>0.98774057474294752</v>
+      </c>
+    </row>
+    <row r="5" spans="1:7">
+      <c r="A5" t="s">
+        <v>458</v>
+      </c>
+      <c r="B5">
+        <v>1</v>
+      </c>
+      <c r="C5" t="s">
+        <v>211</v>
+      </c>
+      <c r="D5">
+        <v>4</v>
+      </c>
+      <c r="E5">
+        <v>7586</v>
+      </c>
+      <c r="F5">
+        <v>7510</v>
+      </c>
+      <c r="G5" s="4">
+        <f t="shared" si="0"/>
+        <v>0.98998154495122592</v>
+      </c>
+    </row>
+    <row r="6" spans="1:7">
+      <c r="A6" t="s">
+        <v>458</v>
+      </c>
+      <c r="B6">
+        <v>2</v>
+      </c>
+      <c r="C6" t="s">
+        <v>449</v>
+      </c>
+      <c r="D6">
+        <v>1</v>
+      </c>
+      <c r="E6">
+        <v>1188</v>
+      </c>
+      <c r="F6">
+        <v>503</v>
+      </c>
+      <c r="G6" s="4">
+        <f t="shared" si="0"/>
+        <v>0.42340067340067339</v>
+      </c>
+    </row>
+    <row r="7" spans="1:7">
+      <c r="A7" t="s">
+        <v>458</v>
+      </c>
+      <c r="B7">
+        <v>2</v>
+      </c>
+      <c r="C7" t="s">
+        <v>459</v>
+      </c>
+      <c r="D7">
+        <v>2</v>
+      </c>
+      <c r="E7">
+        <v>1188</v>
+      </c>
+      <c r="F7">
+        <v>672</v>
+      </c>
+      <c r="G7" s="4">
+        <f t="shared" si="0"/>
+        <v>0.56565656565656564</v>
+      </c>
+    </row>
+    <row r="8" spans="1:7">
+      <c r="A8" t="s">
+        <v>458</v>
+      </c>
+      <c r="B8">
+        <v>2</v>
+      </c>
+      <c r="C8" t="s">
+        <v>460</v>
+      </c>
+      <c r="D8">
+        <v>3</v>
+      </c>
+      <c r="E8">
+        <v>1188</v>
+      </c>
+      <c r="F8">
+        <v>766</v>
+      </c>
+      <c r="G8" s="4">
+        <f t="shared" si="0"/>
+        <v>0.64478114478114479</v>
+      </c>
+    </row>
+    <row r="9" spans="1:7">
+      <c r="A9" t="s">
+        <v>458</v>
+      </c>
+      <c r="B9">
+        <v>2</v>
+      </c>
+      <c r="C9" t="s">
+        <v>461</v>
+      </c>
+      <c r="D9">
+        <v>4</v>
+      </c>
+      <c r="E9">
+        <v>1188</v>
+      </c>
+      <c r="F9">
+        <v>812</v>
+      </c>
+      <c r="G9" s="4">
+        <f t="shared" si="0"/>
+        <v>0.6835016835016835</v>
+      </c>
+    </row>
+    <row r="10" spans="1:7">
+      <c r="A10" t="s">
+        <v>458</v>
+      </c>
+      <c r="B10">
+        <v>2</v>
+      </c>
+      <c r="C10" t="s">
+        <v>463</v>
+      </c>
+      <c r="D10">
+        <v>5</v>
+      </c>
+      <c r="E10">
+        <v>1188</v>
+      </c>
+      <c r="F10">
+        <v>901</v>
+      </c>
+      <c r="G10" s="4">
+        <f t="shared" si="0"/>
+        <v>0.75841750841750843</v>
+      </c>
+    </row>
+    <row r="11" spans="1:7">
+      <c r="A11" t="s">
+        <v>458</v>
+      </c>
+      <c r="B11">
+        <v>2</v>
+      </c>
+      <c r="C11" t="s">
+        <v>462</v>
+      </c>
+      <c r="D11">
+        <v>6</v>
+      </c>
+      <c r="E11">
+        <v>1188</v>
+      </c>
+      <c r="F11">
+        <v>915</v>
+      </c>
+      <c r="G11" s="4">
+        <f t="shared" si="0"/>
+        <v>0.77020202020202022</v>
+      </c>
+    </row>
+    <row r="12" spans="1:7">
+      <c r="A12" t="s">
+        <v>458</v>
+      </c>
+      <c r="B12">
+        <v>2</v>
+      </c>
+      <c r="C12" t="s">
+        <v>464</v>
+      </c>
+      <c r="D12">
+        <v>7</v>
+      </c>
+      <c r="E12">
+        <v>1188</v>
+      </c>
+      <c r="F12">
+        <v>916</v>
+      </c>
+      <c r="G12" s="4">
+        <f t="shared" si="0"/>
+        <v>0.77104377104377109</v>
+      </c>
+    </row>
+    <row r="13" spans="1:7">
+      <c r="A13" t="s">
+        <v>458</v>
+      </c>
+      <c r="B13">
+        <v>2</v>
+      </c>
+      <c r="C13" t="s">
+        <v>465</v>
+      </c>
+      <c r="D13">
+        <v>8</v>
+      </c>
+      <c r="E13">
+        <v>1188</v>
+      </c>
+      <c r="F13">
+        <v>990</v>
+      </c>
+      <c r="G13" s="4">
+        <f t="shared" si="0"/>
+        <v>0.83333333333333337</v>
+      </c>
+    </row>
+    <row r="14" spans="1:7">
+      <c r="A14" t="s">
+        <v>458</v>
+      </c>
+      <c r="B14">
+        <v>2</v>
+      </c>
+      <c r="C14" t="s">
+        <v>466</v>
+      </c>
+      <c r="D14">
+        <v>9</v>
+      </c>
+      <c r="E14">
+        <v>1188</v>
+      </c>
+      <c r="F14">
+        <v>997</v>
+      </c>
+      <c r="G14" s="4">
+        <f t="shared" si="0"/>
+        <v>0.83922558922558921</v>
+      </c>
+    </row>
+    <row r="15" spans="1:7">
+      <c r="A15" t="s">
+        <v>458</v>
+      </c>
+      <c r="B15">
+        <v>2</v>
+      </c>
+      <c r="C15" t="s">
+        <v>468</v>
+      </c>
+      <c r="D15">
+        <v>10</v>
+      </c>
+      <c r="E15">
+        <v>1188</v>
+      </c>
+      <c r="F15">
+        <v>1013</v>
+      </c>
+      <c r="G15" s="4">
+        <f t="shared" si="0"/>
+        <v>0.85269360269360273</v>
+      </c>
+    </row>
+    <row r="16" spans="1:7">
+      <c r="A16" t="s">
+        <v>458</v>
+      </c>
+      <c r="B16">
+        <v>2</v>
+      </c>
+      <c r="C16" t="s">
+        <v>467</v>
+      </c>
+      <c r="D16">
+        <v>11</v>
+      </c>
+      <c r="E16">
+        <v>1188</v>
+      </c>
+      <c r="F16">
+        <v>1014</v>
+      </c>
+      <c r="G16" s="4">
+        <f t="shared" si="0"/>
+        <v>0.85353535353535348</v>
+      </c>
+    </row>
+    <row r="17" spans="1:7">
+      <c r="A17" t="s">
+        <v>458</v>
+      </c>
+      <c r="B17">
+        <v>2</v>
+      </c>
+      <c r="C17" t="s">
+        <v>469</v>
+      </c>
+      <c r="D17">
+        <v>12</v>
+      </c>
+      <c r="E17">
+        <v>1188</v>
+      </c>
+      <c r="F17">
+        <v>1084</v>
+      </c>
+      <c r="G17" s="4">
+        <f t="shared" si="0"/>
+        <v>0.91245791245791241</v>
+      </c>
+    </row>
+    <row r="18" spans="1:7">
+      <c r="A18" t="s">
+        <v>458</v>
+      </c>
+      <c r="B18">
+        <v>2</v>
+      </c>
+      <c r="C18" t="s">
+        <v>470</v>
+      </c>
+      <c r="D18">
+        <v>13</v>
+      </c>
+      <c r="E18">
+        <v>1188</v>
+      </c>
+      <c r="F18">
+        <v>1086</v>
+      </c>
+      <c r="G18" s="4">
+        <f t="shared" si="0"/>
+        <v>0.91414141414141414</v>
+      </c>
+    </row>
+    <row r="19" spans="1:7">
+      <c r="A19" t="s">
+        <v>458</v>
+      </c>
+      <c r="B19">
+        <v>2</v>
+      </c>
+      <c r="C19" t="s">
+        <v>471</v>
+      </c>
+      <c r="D19">
+        <v>14</v>
+      </c>
+      <c r="E19">
+        <v>1188</v>
+      </c>
+      <c r="F19">
+        <v>1094</v>
+      </c>
+      <c r="G19" s="4">
+        <f t="shared" si="0"/>
+        <v>0.92087542087542085</v>
+      </c>
+    </row>
+    <row r="20" spans="1:7">
+      <c r="A20" t="s">
+        <v>458</v>
+      </c>
+      <c r="B20">
+        <v>2</v>
+      </c>
+      <c r="C20" t="s">
+        <v>472</v>
+      </c>
+      <c r="D20">
+        <v>15</v>
+      </c>
+      <c r="E20">
+        <v>1188</v>
+      </c>
+      <c r="F20">
+        <v>1171</v>
+      </c>
+      <c r="G20" s="4">
+        <f t="shared" si="0"/>
+        <v>0.98569023569023573</v>
+      </c>
+    </row>
+    <row r="21" spans="1:7">
+      <c r="A21" t="s">
+        <v>458</v>
+      </c>
+      <c r="B21">
+        <v>6</v>
+      </c>
+      <c r="C21" t="s">
+        <v>473</v>
+      </c>
+      <c r="D21">
+        <v>1</v>
+      </c>
+      <c r="E21">
+        <v>666</v>
+      </c>
+      <c r="F21">
+        <v>104</v>
+      </c>
+      <c r="G21" s="4">
+        <f t="shared" si="0"/>
+        <v>0.15615615615615616</v>
+      </c>
+    </row>
+    <row r="22" spans="1:7">
+      <c r="A22" t="s">
+        <v>458</v>
+      </c>
+      <c r="B22">
+        <v>6</v>
+      </c>
+      <c r="C22" t="s">
+        <v>448</v>
+      </c>
+      <c r="D22">
+        <v>2</v>
+      </c>
+      <c r="E22">
+        <v>666</v>
+      </c>
+      <c r="F22">
+        <v>198</v>
+      </c>
+      <c r="G22" s="4">
+        <f t="shared" si="0"/>
+        <v>0.29729729729729731</v>
+      </c>
+    </row>
+    <row r="23" spans="1:7">
+      <c r="A23" t="s">
+        <v>458</v>
+      </c>
+      <c r="B23">
+        <v>6</v>
+      </c>
+      <c r="C23" t="s">
+        <v>474</v>
+      </c>
+      <c r="D23">
+        <v>3</v>
+      </c>
+      <c r="E23">
+        <v>666</v>
+      </c>
+      <c r="F23">
+        <v>468</v>
+      </c>
+      <c r="G23" s="4">
+        <f t="shared" si="0"/>
+        <v>0.70270270270270274</v>
+      </c>
+    </row>
+    <row r="24" spans="1:7">
+      <c r="A24" t="s">
+        <v>458</v>
+      </c>
+      <c r="B24">
+        <v>6</v>
+      </c>
+      <c r="C24" t="s">
+        <v>485</v>
+      </c>
+      <c r="D24">
+        <v>4</v>
+      </c>
+      <c r="E24">
+        <v>666</v>
+      </c>
+      <c r="F24">
+        <v>1990</v>
+      </c>
+      <c r="G24" s="4">
+        <f t="shared" si="0"/>
+        <v>2.9879879879879878</v>
+      </c>
+    </row>
+    <row r="25" spans="1:7">
+      <c r="A25" t="s">
+        <v>458</v>
+      </c>
+      <c r="B25">
+        <v>6</v>
+      </c>
+      <c r="C25" t="s">
+        <v>475</v>
+      </c>
+      <c r="D25">
+        <v>5</v>
+      </c>
+      <c r="E25">
+        <v>666</v>
+      </c>
+      <c r="F25">
+        <v>2637</v>
+      </c>
+      <c r="G25" s="4">
+        <f t="shared" si="0"/>
+        <v>3.9594594594594597</v>
+      </c>
+    </row>
+    <row r="26" spans="1:7">
+      <c r="A26" t="s">
+        <v>458</v>
+      </c>
+      <c r="B26">
+        <v>9</v>
+      </c>
+      <c r="C26" t="s">
+        <v>477</v>
+      </c>
+      <c r="D26">
+        <v>1</v>
+      </c>
+      <c r="E26">
+        <v>2157</v>
+      </c>
+      <c r="F26">
+        <v>163</v>
+      </c>
+      <c r="G26" s="4">
+        <f t="shared" si="0"/>
+        <v>7.5567918405192391E-2</v>
+      </c>
+    </row>
+    <row r="27" spans="1:7">
+      <c r="A27" t="s">
+        <v>458</v>
+      </c>
+      <c r="B27">
+        <v>9</v>
+      </c>
+      <c r="C27" t="s">
+        <v>478</v>
+      </c>
+      <c r="D27">
+        <v>2</v>
+      </c>
+      <c r="E27">
+        <v>2157</v>
+      </c>
+      <c r="F27">
+        <v>164</v>
+      </c>
+      <c r="G27" s="4">
+        <f t="shared" si="0"/>
+        <v>7.6031525266573946E-2</v>
+      </c>
+    </row>
+    <row r="28" spans="1:7">
+      <c r="A28" t="s">
+        <v>458</v>
+      </c>
+      <c r="B28">
+        <v>9</v>
+      </c>
+      <c r="C28" t="s">
+        <v>476</v>
+      </c>
+      <c r="D28">
+        <v>3</v>
+      </c>
+      <c r="E28">
+        <v>2157</v>
+      </c>
+      <c r="F28">
+        <v>168</v>
+      </c>
+      <c r="G28" s="4">
+        <f t="shared" si="0"/>
+        <v>7.7885952712100137E-2</v>
+      </c>
+    </row>
+    <row r="29" spans="1:7">
+      <c r="A29" t="s">
+        <v>458</v>
+      </c>
+      <c r="B29">
+        <v>9</v>
+      </c>
+      <c r="C29" t="s">
+        <v>479</v>
+      </c>
+      <c r="D29">
+        <v>4</v>
+      </c>
+      <c r="E29">
+        <v>2157</v>
+      </c>
+      <c r="F29">
+        <v>351</v>
+      </c>
+      <c r="G29" s="4">
+        <f t="shared" si="0"/>
+        <v>0.16272600834492351</v>
+      </c>
+    </row>
+    <row r="30" spans="1:7">
+      <c r="A30" t="s">
+        <v>458</v>
+      </c>
+      <c r="B30">
+        <v>9</v>
+      </c>
+      <c r="C30" t="s">
+        <v>449</v>
+      </c>
+      <c r="D30">
+        <v>5</v>
+      </c>
+      <c r="E30">
+        <v>2157</v>
+      </c>
+      <c r="F30">
+        <v>354</v>
+      </c>
+      <c r="G30" s="4">
+        <f t="shared" si="0"/>
+        <v>0.16411682892906815</v>
+      </c>
+    </row>
+    <row r="31" spans="1:7">
+      <c r="A31" t="s">
+        <v>458</v>
+      </c>
+      <c r="B31">
+        <v>9</v>
+      </c>
+      <c r="C31" t="s">
+        <v>480</v>
+      </c>
+      <c r="D31">
+        <v>6</v>
+      </c>
+      <c r="E31">
+        <v>2157</v>
+      </c>
+      <c r="F31">
+        <v>731</v>
+      </c>
+      <c r="G31" s="4">
+        <f t="shared" si="0"/>
+        <v>0.33889661566991192</v>
+      </c>
+    </row>
+    <row r="32" spans="1:7">
+      <c r="A32" t="s">
+        <v>458</v>
+      </c>
+      <c r="B32">
+        <v>9</v>
+      </c>
+      <c r="C32" t="s">
+        <v>481</v>
+      </c>
+      <c r="D32">
+        <v>7</v>
+      </c>
+      <c r="E32">
+        <v>2157</v>
+      </c>
+      <c r="F32">
+        <v>736</v>
+      </c>
+      <c r="G32" s="4">
+        <f t="shared" si="0"/>
+        <v>0.34121464997681966</v>
+      </c>
+    </row>
+    <row r="33" spans="1:7">
+      <c r="A33" t="s">
+        <v>458</v>
+      </c>
+      <c r="B33">
+        <v>9</v>
+      </c>
+      <c r="C33" t="s">
+        <v>482</v>
+      </c>
+      <c r="D33">
+        <v>8</v>
+      </c>
+      <c r="E33">
+        <v>2157</v>
+      </c>
+      <c r="F33">
+        <v>752</v>
+      </c>
+      <c r="G33" s="4">
+        <f t="shared" si="0"/>
+        <v>0.34863235975892443</v>
+      </c>
+    </row>
+    <row r="34" spans="1:7">
+      <c r="A34" t="s">
+        <v>458</v>
+      </c>
+      <c r="B34">
+        <v>9</v>
+      </c>
+      <c r="C34" t="s">
+        <v>483</v>
+      </c>
+      <c r="D34">
+        <v>9</v>
+      </c>
+      <c r="E34">
+        <v>2157</v>
+      </c>
+      <c r="F34">
+        <v>883</v>
+      </c>
+      <c r="G34" s="4">
+        <f t="shared" si="0"/>
+        <v>0.40936485859990729</v>
+      </c>
+    </row>
+    <row r="35" spans="1:7">
+      <c r="A35" t="s">
+        <v>458</v>
+      </c>
+      <c r="B35">
+        <v>9</v>
+      </c>
+      <c r="C35" t="s">
+        <v>484</v>
+      </c>
+      <c r="D35">
+        <v>10</v>
+      </c>
+      <c r="E35">
+        <v>2157</v>
+      </c>
+      <c r="F35">
+        <v>886</v>
+      </c>
+      <c r="G35" s="4">
+        <f t="shared" si="0"/>
+        <v>0.41075567918405193</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <extLst>
+    <ext xmlns:mx="http://schemas.microsoft.com/office/mac/excel/2008/main" uri="{64002731-A6B0-56B0-2670-7721B7C09600}">
+      <mx:PLV Mode="0" OnePage="0" WScale="0"/>
+    </ext>
+  </extLst>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+  <dimension ref="A1:G1"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0"/>
+  <sheetData>
+    <row r="1" spans="1:7">
+      <c r="A1" t="s">
+        <v>270</v>
+      </c>
+      <c r="B1" t="s">
+        <v>272</v>
+      </c>
+      <c r="C1" t="s">
+        <v>446</v>
+      </c>
+      <c r="D1" s="2" t="s">
+        <v>450</v>
+      </c>
+      <c r="E1" s="2" t="s">
+        <v>452</v>
+      </c>
+      <c r="F1" s="2" t="s">
+        <v>451</v>
+      </c>
+      <c r="G1" s="2" t="s">
+        <v>453</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <extLst>
+    <ext xmlns:mx="http://schemas.microsoft.com/office/mac/excel/2008/main" uri="{64002731-A6B0-56B0-2670-7721B7C09600}">
+      <mx:PLV Mode="0" OnePage="0" WScale="0"/>
+    </ext>
+  </extLst>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+  <dimension ref="A1:B5"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0"/>
+  <cols>
+    <col min="1" max="1" width="12.33203125" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:2">
+      <c r="A1" s="2" t="s">
+        <v>432</v>
+      </c>
+      <c r="B1" s="2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="2" spans="1:2">
+      <c r="A2" s="2" t="s">
+        <v>432</v>
+      </c>
+      <c r="B2" s="2">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="3" spans="1:2">
+      <c r="A3" s="2" t="s">
+        <v>432</v>
+      </c>
+      <c r="B3" s="2">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="4" spans="1:2">
+      <c r="A4" s="2" t="s">
+        <v>432</v>
+      </c>
+      <c r="B4" s="2">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="5" spans="1:2">
+      <c r="A5" s="2" t="s">
+        <v>432</v>
+      </c>
+      <c r="B5" s="2">
+        <v>9</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <pageSetup orientation="portrait" horizontalDpi="4294967292" verticalDpi="4294967292"/>
+  <extLst>
+    <ext xmlns:mx="http://schemas.microsoft.com/office/mac/excel/2008/main" uri="{64002731-A6B0-56B0-2670-7721B7C09600}">
+      <mx:PLV Mode="0" OnePage="0" WScale="0"/>
+    </ext>
+  </extLst>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
fresh results without loops
</commit_message>
<xml_diff>
--- a/ScratchData/data.xlsx
+++ b/ScratchData/data.xlsx
@@ -4,7 +4,7 @@
   <fileVersion appName="xl" lastEdited="5" lowestEdited="5" rupBuild="28125"/>
   <workbookPr showInkAnnotation="0" autoCompressPictures="0"/>
   <bookViews>
-    <workbookView xWindow="2800" yWindow="0" windowWidth="28420" windowHeight="17740" tabRatio="680" firstSheet="2" activeTab="3"/>
+    <workbookView xWindow="9580" yWindow="100" windowWidth="28420" windowHeight="17740" tabRatio="680" firstSheet="2" activeTab="3"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -30,7 +30,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3820" uniqueCount="970">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3816" uniqueCount="972">
   <si>
     <t>Done in 748</t>
   </si>
@@ -2940,6 +2940,12 @@
   </si>
   <si>
     <t>over 50% info</t>
+  </si>
+  <si>
+    <t>test.Class11_7_</t>
+  </si>
+  <si>
+    <t>there need to collect it</t>
   </si>
 </sst>
 </file>
@@ -3007,8 +3013,12 @@
       <diagonal/>
     </border>
   </borders>
-  <cellStyleXfs count="173">
+  <cellStyleXfs count="177">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
@@ -3195,7 +3205,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
   </cellXfs>
-  <cellStyles count="173">
+  <cellStyles count="177">
     <cellStyle name="Followed Hyperlink" xfId="2" builtinId="9" hidden="1"/>
     <cellStyle name="Followed Hyperlink" xfId="4" builtinId="9" hidden="1"/>
     <cellStyle name="Followed Hyperlink" xfId="6" builtinId="9" hidden="1"/>
@@ -3282,6 +3292,8 @@
     <cellStyle name="Followed Hyperlink" xfId="168" builtinId="9" hidden="1"/>
     <cellStyle name="Followed Hyperlink" xfId="170" builtinId="9" hidden="1"/>
     <cellStyle name="Followed Hyperlink" xfId="172" builtinId="9" hidden="1"/>
+    <cellStyle name="Followed Hyperlink" xfId="174" builtinId="9" hidden="1"/>
+    <cellStyle name="Followed Hyperlink" xfId="176" builtinId="9" hidden="1"/>
     <cellStyle name="Hyperlink" xfId="1" builtinId="8" hidden="1"/>
     <cellStyle name="Hyperlink" xfId="3" builtinId="8" hidden="1"/>
     <cellStyle name="Hyperlink" xfId="5" builtinId="8" hidden="1"/>
@@ -3368,6 +3380,8 @@
     <cellStyle name="Hyperlink" xfId="167" builtinId="8" hidden="1"/>
     <cellStyle name="Hyperlink" xfId="169" builtinId="8" hidden="1"/>
     <cellStyle name="Hyperlink" xfId="171" builtinId="8" hidden="1"/>
+    <cellStyle name="Hyperlink" xfId="173" builtinId="8" hidden="1"/>
+    <cellStyle name="Hyperlink" xfId="175" builtinId="8" hidden="1"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
@@ -3860,16 +3874,16 @@
                 <c:formatCode>0</c:formatCode>
                 <c:ptCount val="6"/>
                 <c:pt idx="0">
-                  <c:v>30.0</c:v>
+                  <c:v>31.0</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>19.0</c:v>
+                  <c:v>20.0</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>13.0</c:v>
+                  <c:v>14.0</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>9.0</c:v>
+                  <c:v>10.0</c:v>
                 </c:pt>
                 <c:pt idx="4">
                   <c:v>1.0</c:v>
@@ -4217,10 +4231,10 @@
                   <c:v>25.0</c:v>
                 </c:pt>
                 <c:pt idx="4">
-                  <c:v>60.0</c:v>
+                  <c:v>61.0</c:v>
                 </c:pt>
                 <c:pt idx="5">
-                  <c:v>62.0</c:v>
+                  <c:v>63.0</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -11966,28 +11980,28 @@
       </c>
     </row>
     <row r="159" spans="1:9">
-      <c r="A159" t="s">
+      <c r="A159" s="6" t="s">
         <v>489</v>
       </c>
-      <c r="B159">
+      <c r="B159" s="6">
         <v>20</v>
       </c>
-      <c r="C159">
+      <c r="C159" s="6">
         <v>33</v>
       </c>
-      <c r="D159">
+      <c r="D159" s="6">
         <v>101</v>
       </c>
-      <c r="E159">
-        <v>0</v>
-      </c>
-      <c r="F159">
+      <c r="E159" s="6">
+        <v>0</v>
+      </c>
+      <c r="F159" s="6">
         <v>4</v>
       </c>
-      <c r="G159">
-        <v>0</v>
-      </c>
-      <c r="H159">
+      <c r="G159" s="6">
+        <v>0</v>
+      </c>
+      <c r="H159" s="6">
         <v>101</v>
       </c>
       <c r="I159" s="4">
@@ -23897,7 +23911,7 @@
 
 <file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:CI540"/>
+  <dimension ref="A1:CJ540"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0"/>
   <cols>
     <col min="3" max="3" width="28.5" bestFit="1" customWidth="1"/>
@@ -23906,7 +23920,7 @@
     <col min="35" max="35" width="13" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:87">
+    <row r="1" spans="1:88">
       <c r="A1" t="s">
         <v>486</v>
       </c>
@@ -24149,8 +24163,11 @@
       <c r="CI1" t="s">
         <v>894</v>
       </c>
-    </row>
-    <row r="2" spans="1:87">
+      <c r="CJ1" t="s">
+        <v>894</v>
+      </c>
+    </row>
+    <row r="2" spans="1:88">
       <c r="A2" t="s">
         <v>458</v>
       </c>
@@ -24223,8 +24240,8 @@
         <v>895</v>
       </c>
       <c r="W2">
-        <f>COUNTA(X2:CI2)</f>
-        <v>64</v>
+        <f>COUNTA(X2:CJ2)</f>
+        <v>65</v>
       </c>
       <c r="X2" t="s">
         <v>905</v>
@@ -24269,157 +24286,160 @@
         <v>902</v>
       </c>
       <c r="AL2" t="s">
+        <v>970</v>
+      </c>
+      <c r="AM2" t="s">
         <v>904</v>
       </c>
-      <c r="AM2" t="s">
+      <c r="AN2" t="s">
         <v>916</v>
       </c>
-      <c r="AN2" t="s">
+      <c r="AO2" t="s">
         <v>917</v>
       </c>
-      <c r="AO2" t="s">
+      <c r="AP2" t="s">
         <v>918</v>
       </c>
-      <c r="AP2" t="s">
+      <c r="AQ2" t="s">
         <v>919</v>
       </c>
-      <c r="AQ2" t="s">
+      <c r="AR2" t="s">
         <v>920</v>
       </c>
-      <c r="AR2" t="s">
+      <c r="AS2" t="s">
         <v>921</v>
       </c>
-      <c r="AS2" t="s">
+      <c r="AT2" t="s">
         <v>922</v>
       </c>
-      <c r="AT2" t="s">
+      <c r="AU2" t="s">
         <v>923</v>
       </c>
-      <c r="AU2" t="s">
+      <c r="AV2" t="s">
         <v>924</v>
       </c>
-      <c r="AV2" t="s">
+      <c r="AW2" t="s">
         <v>925</v>
       </c>
-      <c r="AW2" t="s">
+      <c r="AX2" t="s">
         <v>926</v>
       </c>
-      <c r="AX2" t="s">
+      <c r="AY2" t="s">
         <v>927</v>
       </c>
-      <c r="AY2" t="s">
+      <c r="AZ2" t="s">
         <v>928</v>
       </c>
-      <c r="AZ2" t="s">
+      <c r="BA2" t="s">
         <v>929</v>
       </c>
-      <c r="BA2" t="s">
+      <c r="BB2" t="s">
         <v>930</v>
       </c>
-      <c r="BB2" t="s">
+      <c r="BC2" t="s">
         <v>931</v>
       </c>
-      <c r="BC2" t="s">
+      <c r="BD2" t="s">
         <v>932</v>
       </c>
-      <c r="BD2" t="s">
+      <c r="BE2" t="s">
         <v>933</v>
       </c>
-      <c r="BE2" t="s">
+      <c r="BF2" t="s">
         <v>934</v>
       </c>
-      <c r="BF2" t="s">
+      <c r="BG2" t="s">
         <v>935</v>
       </c>
-      <c r="BG2" t="s">
+      <c r="BH2" t="s">
         <v>936</v>
       </c>
-      <c r="BH2" t="s">
+      <c r="BI2" t="s">
         <v>937</v>
       </c>
-      <c r="BI2" t="s">
+      <c r="BJ2" t="s">
         <v>938</v>
       </c>
-      <c r="BJ2" t="s">
+      <c r="BK2" t="s">
         <v>939</v>
       </c>
-      <c r="BK2" t="s">
+      <c r="BL2" t="s">
         <v>940</v>
       </c>
-      <c r="BL2" t="s">
+      <c r="BM2" t="s">
         <v>941</v>
       </c>
-      <c r="BM2" t="s">
+      <c r="BN2" t="s">
         <v>942</v>
       </c>
-      <c r="BN2" t="s">
+      <c r="BO2" t="s">
         <v>943</v>
       </c>
-      <c r="BO2" t="s">
+      <c r="BP2" t="s">
         <v>944</v>
       </c>
-      <c r="BP2" t="s">
+      <c r="BQ2" t="s">
         <v>945</v>
       </c>
-      <c r="BQ2" t="s">
+      <c r="BR2" t="s">
         <v>946</v>
       </c>
-      <c r="BR2" t="s">
+      <c r="BS2" t="s">
         <v>947</v>
       </c>
-      <c r="BS2" t="s">
+      <c r="BT2" t="s">
         <v>948</v>
       </c>
-      <c r="BT2" t="s">
+      <c r="BU2" t="s">
         <v>949</v>
       </c>
-      <c r="BU2" t="s">
+      <c r="BV2" t="s">
         <v>950</v>
       </c>
-      <c r="BV2" t="s">
+      <c r="BW2" t="s">
         <v>951</v>
       </c>
-      <c r="BW2" t="s">
+      <c r="BX2" t="s">
         <v>952</v>
       </c>
-      <c r="BX2" t="s">
+      <c r="BY2" t="s">
         <v>953</v>
       </c>
-      <c r="BY2" t="s">
+      <c r="BZ2" t="s">
         <v>954</v>
       </c>
-      <c r="BZ2" t="s">
+      <c r="CA2" t="s">
         <v>955</v>
       </c>
-      <c r="CA2" t="s">
+      <c r="CB2" t="s">
         <v>956</v>
       </c>
-      <c r="CB2" t="s">
+      <c r="CC2" t="s">
         <v>957</v>
       </c>
-      <c r="CC2" t="s">
+      <c r="CD2" t="s">
         <v>958</v>
       </c>
-      <c r="CD2" t="s">
+      <c r="CE2" t="s">
         <v>959</v>
       </c>
-      <c r="CE2" t="s">
+      <c r="CF2" t="s">
         <v>960</v>
       </c>
-      <c r="CF2" t="s">
+      <c r="CG2" t="s">
         <v>961</v>
       </c>
-      <c r="CG2" t="s">
+      <c r="CH2" t="s">
         <v>962</v>
       </c>
-      <c r="CH2" t="s">
+      <c r="CI2" t="s">
         <v>963</v>
       </c>
-      <c r="CI2" t="s">
+      <c r="CJ2" t="s">
         <v>964</v>
       </c>
     </row>
-    <row r="3" spans="1:87">
+    <row r="3" spans="1:88">
       <c r="A3" t="s">
         <v>458</v>
       </c>
@@ -24470,33 +24490,33 @@
       </c>
       <c r="O3" s="4">
         <f>SUM(Q3:V3)</f>
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="P3" t="s">
         <v>890</v>
       </c>
       <c r="Q3" s="8">
-        <f>COUNTIF($X3:$CI3,"=0")</f>
-        <v>30</v>
+        <f>COUNTIF($X3:$CJ3,"=0")</f>
+        <v>31</v>
       </c>
       <c r="R3" s="8">
-        <f>COUNTIFS($X3:$CI3,"&gt;0",$X3:$CI3,"&lt;0.25")</f>
+        <f>COUNTIFS($X3:$CJ3,"&gt;0",$X3:$CJ3,"&lt;0.25")</f>
         <v>21</v>
       </c>
       <c r="S3" s="8">
-        <f>COUNTIFS($X3:$CI3,"&gt;=0.25",$X3:$CI3,"&lt;0.5")</f>
+        <f>COUNTIFS($X3:$CJ3,"&gt;=0.25",$X3:$CJ3,"&lt;0.5")</f>
         <v>7</v>
       </c>
       <c r="T3" s="8">
-        <f>COUNTIFS($X3:$CI3,"&gt;=0.5",$X3:$CI3,"&lt;0.75")</f>
+        <f>COUNTIFS($X3:$CJ3,"&gt;=0.5",$X3:$CJ3,"&lt;0.75")</f>
         <v>5</v>
       </c>
       <c r="U3" s="8">
-        <f>COUNTIFS($X3:$CI3,"&gt;=0.75",$X3:$CI3,"&lt;1")</f>
+        <f>COUNTIFS($X3:$CJ3,"&gt;=0.75",$X3:$CJ3,"&lt;1")</f>
         <v>1</v>
       </c>
       <c r="V3" s="8">
-        <f>COUNTIF($X3:$CI3,"=1")</f>
+        <f>COUNTIF($X3:$CJ3,"=1")</f>
         <v>0</v>
       </c>
       <c r="W3" t="s">
@@ -24560,27 +24580,27 @@
       </c>
       <c r="AL3">
         <f>DMAX($A$1:$L$540,$W3,AL$1:AL$2)</f>
-        <v>0.58620689655172409</v>
+        <v>0</v>
       </c>
       <c r="AM3">
         <f>DMAX($A$1:$L$540,$W3,AM$1:AM$2)</f>
-        <v>0.11979166666666667</v>
+        <v>0.58620689655172409</v>
       </c>
       <c r="AN3">
         <f>DMAX($A$1:$L$540,$W3,AN$1:AN$2)</f>
-        <v>8.4745762711864406E-3</v>
+        <v>0.11979166666666667</v>
       </c>
       <c r="AO3">
         <f>DMAX($A$1:$L$540,$W3,AO$1:AO$2)</f>
-        <v>0</v>
+        <v>8.4745762711864406E-3</v>
       </c>
       <c r="AP3">
         <f>DMAX($A$1:$L$540,$W3,AP$1:AP$2)</f>
-        <v>0.24848484848484848</v>
+        <v>0</v>
       </c>
       <c r="AQ3">
         <f>DMAX($A$1:$L$540,$W3,AQ$1:AQ$2)</f>
-        <v>0</v>
+        <v>0.24848484848484848</v>
       </c>
       <c r="AR3">
         <f>DMAX($A$1:$L$540,$W3,AR$1:AR$2)</f>
@@ -24592,87 +24612,87 @@
       </c>
       <c r="AT3">
         <f>DMAX($A$1:$L$540,$W3,AT$1:AT$2)</f>
-        <v>7.3170731707317069E-2</v>
+        <v>0</v>
       </c>
       <c r="AU3">
         <f>DMAX($A$1:$L$540,$W3,AU$1:AU$2)</f>
-        <v>9.6774193548387094E-2</v>
+        <v>7.3170731707317069E-2</v>
       </c>
       <c r="AV3">
         <f>DMAX($A$1:$L$540,$W3,AV$1:AV$2)</f>
-        <v>0.5178571428571429</v>
+        <v>9.6774193548387094E-2</v>
       </c>
       <c r="AW3">
         <f>DMAX($A$1:$L$540,$W3,AW$1:AW$2)</f>
-        <v>0.36046511627906974</v>
+        <v>0.5178571428571429</v>
       </c>
       <c r="AX3">
         <f>DMAX($A$1:$L$540,$W3,AX$1:AX$2)</f>
-        <v>0.19565217391304349</v>
+        <v>0.36046511627906974</v>
       </c>
       <c r="AY3">
         <f>DMAX($A$1:$L$540,$W3,AY$1:AY$2)</f>
-        <v>3.3333333333333333E-2</v>
+        <v>0.19565217391304349</v>
       </c>
       <c r="AZ3">
         <f>DMAX($A$1:$L$540,$W3,AZ$1:AZ$2)</f>
-        <v>0</v>
+        <v>3.3333333333333333E-2</v>
       </c>
       <c r="BA3">
         <f>DMAX($A$1:$L$540,$W3,BA$1:BA$2)</f>
-        <v>0.23214285714285715</v>
+        <v>0</v>
       </c>
       <c r="BB3">
         <f>DMAX($A$1:$L$540,$W3,BB$1:BB$2)</f>
-        <v>0.2</v>
+        <v>0.23214285714285715</v>
       </c>
       <c r="BC3">
         <f>DMAX($A$1:$L$540,$W3,BC$1:BC$2)</f>
-        <v>0.56617647058823528</v>
+        <v>0.2</v>
       </c>
       <c r="BD3">
         <f>DMAX($A$1:$L$540,$W3,BD$1:BD$2)</f>
-        <v>0</v>
+        <v>0.56617647058823528</v>
       </c>
       <c r="BE3">
         <f>DMAX($A$1:$L$540,$W3,BE$1:BE$2)</f>
-        <v>0.2857142857142857</v>
+        <v>0</v>
       </c>
       <c r="BF3">
         <f>DMAX($A$1:$L$540,$W3,BF$1:BF$2)</f>
-        <v>0</v>
+        <v>0.2857142857142857</v>
       </c>
       <c r="BG3">
         <f>DMAX($A$1:$L$540,$W3,BG$1:BG$2)</f>
-        <v>0.3888888888888889</v>
+        <v>0</v>
       </c>
       <c r="BH3">
         <f>DMAX($A$1:$L$540,$W3,BH$1:BH$2)</f>
-        <v>0.63953488372093026</v>
+        <v>0.3888888888888889</v>
       </c>
       <c r="BI3">
         <f>DMAX($A$1:$L$540,$W3,BI$1:BI$2)</f>
-        <v>0</v>
+        <v>0.63953488372093026</v>
       </c>
       <c r="BJ3">
         <f>DMAX($A$1:$L$540,$W3,BJ$1:BJ$2)</f>
-        <v>0.33962264150943394</v>
+        <v>0</v>
       </c>
       <c r="BK3">
         <f>DMAX($A$1:$L$540,$W3,BK$1:BK$2)</f>
-        <v>6.7842605156037995E-3</v>
+        <v>0.33962264150943394</v>
       </c>
       <c r="BL3">
         <f>DMAX($A$1:$L$540,$W3,BL$1:BL$2)</f>
-        <v>8.4210526315789472E-3</v>
+        <v>6.7842605156037995E-3</v>
       </c>
       <c r="BM3">
         <f>DMAX($A$1:$L$540,$W3,BM$1:BM$2)</f>
-        <v>8.2372322899505763E-3</v>
+        <v>8.4210526315789472E-3</v>
       </c>
       <c r="BN3">
         <f>DMAX($A$1:$L$540,$W3,BN$1:BN$2)</f>
-        <v>0</v>
+        <v>8.2372322899505763E-3</v>
       </c>
       <c r="BO3">
         <f>DMAX($A$1:$L$540,$W3,BO$1:BO$2)</f>
@@ -24684,23 +24704,23 @@
       </c>
       <c r="BQ3">
         <f>DMAX($A$1:$L$540,$W3,BQ$1:BQ$2)</f>
-        <v>0.20408163265306123</v>
+        <v>0</v>
       </c>
       <c r="BR3">
         <f>DMAX($A$1:$L$540,$W3,BR$1:BR$2)</f>
-        <v>0</v>
+        <v>0.20408163265306123</v>
       </c>
       <c r="BS3">
         <f>DMAX($A$1:$L$540,$W3,BS$1:BS$2)</f>
-        <v>0.26548672566371684</v>
+        <v>0</v>
       </c>
       <c r="BT3">
         <f>DMAX($A$1:$L$540,$W3,BT$1:BT$2)</f>
-        <v>0.18085106382978725</v>
+        <v>0.26548672566371684</v>
       </c>
       <c r="BU3">
         <f>DMAX($A$1:$L$540,$W3,BU$1:BU$2)</f>
-        <v>0</v>
+        <v>0.18085106382978725</v>
       </c>
       <c r="BV3">
         <f>DMAX($A$1:$L$540,$W3,BV$1:BV$2)</f>
@@ -24708,15 +24728,15 @@
       </c>
       <c r="BW3">
         <f>DMAX($A$1:$L$540,$W3,BW$1:BW$2)</f>
-        <v>0.27397260273972601</v>
+        <v>0</v>
       </c>
       <c r="BX3">
         <f>DMAX($A$1:$L$540,$W3,BX$1:BX$2)</f>
-        <v>0.31707317073170732</v>
+        <v>0.27397260273972601</v>
       </c>
       <c r="BY3">
         <f>DMAX($A$1:$L$540,$W3,BY$1:BY$2)</f>
-        <v>0</v>
+        <v>0.31707317073170732</v>
       </c>
       <c r="BZ3">
         <f>DMAX($A$1:$L$540,$W3,BZ$1:BZ$2)</f>
@@ -24732,15 +24752,15 @@
       </c>
       <c r="CC3">
         <f>DMAX($A$1:$L$540,$W3,CC$1:CC$2)</f>
-        <v>7.9545454545454544E-2</v>
+        <v>0</v>
       </c>
       <c r="CD3">
         <f>DMAX($A$1:$L$540,$W3,CD$1:CD$2)</f>
-        <v>0.125</v>
+        <v>7.9545454545454544E-2</v>
       </c>
       <c r="CE3">
         <f>DMAX($A$1:$L$540,$W3,CE$1:CE$2)</f>
-        <v>0</v>
+        <v>0.125</v>
       </c>
       <c r="CF3">
         <f>DMAX($A$1:$L$540,$W3,CF$1:CF$2)</f>
@@ -24758,8 +24778,12 @@
         <f>DMAX($A$1:$L$540,$W3,CI$1:CI$2)</f>
         <v>0</v>
       </c>
-    </row>
-    <row r="4" spans="1:87">
+      <c r="CJ3">
+        <f>DMAX($A$1:$L$540,$W3,CJ$1:CJ$2)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="4" spans="1:88">
       <c r="A4" t="s">
         <v>458</v>
       </c>
@@ -24810,33 +24834,33 @@
       </c>
       <c r="O4" s="4">
         <f t="shared" ref="O4:O7" si="8">SUM(Q4:V4)</f>
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="P4" t="s">
         <v>891</v>
       </c>
       <c r="Q4" s="8">
-        <f t="shared" ref="Q4:Q8" si="9">COUNTIF($X4:$CI4,"=0")</f>
-        <v>19</v>
+        <f t="shared" ref="Q4:Q8" si="9">COUNTIF($X4:$CJ4,"=0")</f>
+        <v>20</v>
       </c>
       <c r="R4" s="8">
-        <f t="shared" ref="R4:R8" si="10">COUNTIFS($X4:$CI4,"&gt;0",$X4:$CI4,"&lt;0.25")</f>
+        <f t="shared" ref="R4:R8" si="10">COUNTIFS($X4:$CJ4,"&gt;0",$X4:$CJ4,"&lt;0.25")</f>
         <v>17</v>
       </c>
       <c r="S4" s="8">
-        <f t="shared" ref="S4:S8" si="11">COUNTIFS($X4:$CI4,"&gt;=0.25",$X4:$CI4,"&lt;0.5")</f>
+        <f t="shared" ref="S4:S8" si="11">COUNTIFS($X4:$CJ4,"&gt;=0.25",$X4:$CJ4,"&lt;0.5")</f>
         <v>9</v>
       </c>
       <c r="T4" s="8">
-        <f t="shared" ref="T4:T8" si="12">COUNTIFS($X4:$CI4,"&gt;=0.5",$X4:$CI4,"&lt;0.75")</f>
+        <f t="shared" ref="T4:T8" si="12">COUNTIFS($X4:$CJ4,"&gt;=0.5",$X4:$CJ4,"&lt;0.75")</f>
         <v>10</v>
       </c>
       <c r="U4" s="8">
-        <f t="shared" ref="U4:U8" si="13">COUNTIFS($X4:$CI4,"&gt;=0.75",$X4:$CI4,"&lt;1")</f>
+        <f t="shared" ref="U4:U8" si="13">COUNTIFS($X4:$CJ4,"&gt;=0.75",$X4:$CJ4,"&lt;1")</f>
         <v>3</v>
       </c>
       <c r="V4" s="8">
-        <f t="shared" ref="V4:V8" si="14">COUNTIF($X4:$CI4,"=1")</f>
+        <f t="shared" ref="V4:V8" si="14">COUNTIF($X4:$CJ4,"=1")</f>
         <v>6</v>
       </c>
       <c r="W4" t="s">
@@ -24900,27 +24924,27 @@
       </c>
       <c r="AL4">
         <f>IF(AL3&lt;DMAX($A$1:$L$540,$W4,AL$1:AL$2),DMAX($A$1:$L$540,$W4,AL$1:AL$2),AL3)</f>
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="AM4">
         <f>IF(AM3&lt;DMAX($A$1:$L$540,$W4,AM$1:AM$2),DMAX($A$1:$L$540,$W4,AM$1:AM$2),AM3)</f>
-        <v>0.68229166666666663</v>
+        <v>1</v>
       </c>
       <c r="AN4">
         <f>IF(AN3&lt;DMAX($A$1:$L$540,$W4,AN$1:AN$2),DMAX($A$1:$L$540,$W4,AN$1:AN$2),AN3)</f>
-        <v>8.4745762711864406E-3</v>
+        <v>0.68229166666666663</v>
       </c>
       <c r="AO4">
         <f>IF(AO3&lt;DMAX($A$1:$L$540,$W4,AO$1:AO$2),DMAX($A$1:$L$540,$W4,AO$1:AO$2),AO3)</f>
-        <v>0.20454545454545456</v>
+        <v>8.4745762711864406E-3</v>
       </c>
       <c r="AP4">
         <f>IF(AP3&lt;DMAX($A$1:$L$540,$W4,AP$1:AP$2),DMAX($A$1:$L$540,$W4,AP$1:AP$2),AP3)</f>
-        <v>0.24848484848484848</v>
+        <v>0.20454545454545456</v>
       </c>
       <c r="AQ4">
         <f>IF(AQ3&lt;DMAX($A$1:$L$540,$W4,AQ$1:AQ$2),DMAX($A$1:$L$540,$W4,AQ$1:AQ$2),AQ3)</f>
-        <v>0</v>
+        <v>0.24848484848484848</v>
       </c>
       <c r="AR4">
         <f>IF(AR3&lt;DMAX($A$1:$L$540,$W4,AR$1:AR$2),DMAX($A$1:$L$540,$W4,AR$1:AR$2),AR3)</f>
@@ -24932,87 +24956,87 @@
       </c>
       <c r="AT4">
         <f>IF(AT3&lt;DMAX($A$1:$L$540,$W4,AT$1:AT$2),DMAX($A$1:$L$540,$W4,AT$1:AT$2),AT3)</f>
-        <v>0.14634146341463414</v>
+        <v>0</v>
       </c>
       <c r="AU4">
         <f>IF(AU3&lt;DMAX($A$1:$L$540,$W4,AU$1:AU$2),DMAX($A$1:$L$540,$W4,AU$1:AU$2),AU3)</f>
-        <v>9.6774193548387094E-2</v>
+        <v>0.14634146341463414</v>
       </c>
       <c r="AV4">
         <f>IF(AV3&lt;DMAX($A$1:$L$540,$W4,AV$1:AV$2),DMAX($A$1:$L$540,$W4,AV$1:AV$2),AV3)</f>
-        <v>0.5178571428571429</v>
+        <v>9.6774193548387094E-2</v>
       </c>
       <c r="AW4">
         <f>IF(AW3&lt;DMAX($A$1:$L$540,$W4,AW$1:AW$2),DMAX($A$1:$L$540,$W4,AW$1:AW$2),AW3)</f>
-        <v>0.36046511627906974</v>
+        <v>0.5178571428571429</v>
       </c>
       <c r="AX4">
         <f>IF(AX3&lt;DMAX($A$1:$L$540,$W4,AX$1:AX$2),DMAX($A$1:$L$540,$W4,AX$1:AX$2),AX3)</f>
-        <v>0.45652173913043476</v>
+        <v>0.36046511627906974</v>
       </c>
       <c r="AY4">
         <f>IF(AY3&lt;DMAX($A$1:$L$540,$W4,AY$1:AY$2),DMAX($A$1:$L$540,$W4,AY$1:AY$2),AY3)</f>
-        <v>0.2</v>
+        <v>0.45652173913043476</v>
       </c>
       <c r="AZ4">
         <f>IF(AZ3&lt;DMAX($A$1:$L$540,$W4,AZ$1:AZ$2),DMAX($A$1:$L$540,$W4,AZ$1:AZ$2),AZ3)</f>
-        <v>0</v>
+        <v>0.2</v>
       </c>
       <c r="BA4">
         <f>IF(BA3&lt;DMAX($A$1:$L$540,$W4,BA$1:BA$2),DMAX($A$1:$L$540,$W4,BA$1:BA$2),BA3)</f>
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="BB4">
         <f>IF(BB3&lt;DMAX($A$1:$L$540,$W4,BB$1:BB$2),DMAX($A$1:$L$540,$W4,BB$1:BB$2),BB3)</f>
-        <v>0.8571428571428571</v>
+        <v>1</v>
       </c>
       <c r="BC4">
         <f>IF(BC3&lt;DMAX($A$1:$L$540,$W4,BC$1:BC$2),DMAX($A$1:$L$540,$W4,BC$1:BC$2),BC3)</f>
-        <v>1</v>
+        <v>0.8571428571428571</v>
       </c>
       <c r="BD4">
         <f>IF(BD3&lt;DMAX($A$1:$L$540,$W4,BD$1:BD$2),DMAX($A$1:$L$540,$W4,BD$1:BD$2),BD3)</f>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="BE4">
         <f>IF(BE3&lt;DMAX($A$1:$L$540,$W4,BE$1:BE$2),DMAX($A$1:$L$540,$W4,BE$1:BE$2),BE3)</f>
-        <v>0.47619047619047616</v>
+        <v>0</v>
       </c>
       <c r="BF4">
         <f>IF(BF3&lt;DMAX($A$1:$L$540,$W4,BF$1:BF$2),DMAX($A$1:$L$540,$W4,BF$1:BF$2),BF3)</f>
-        <v>0.73333333333333328</v>
+        <v>0.47619047619047616</v>
       </c>
       <c r="BG4">
         <f>IF(BG3&lt;DMAX($A$1:$L$540,$W4,BG$1:BG$2),DMAX($A$1:$L$540,$W4,BG$1:BG$2),BG3)</f>
-        <v>0.66049382716049387</v>
+        <v>0.73333333333333328</v>
       </c>
       <c r="BH4">
         <f>IF(BH3&lt;DMAX($A$1:$L$540,$W4,BH$1:BH$2),DMAX($A$1:$L$540,$W4,BH$1:BH$2),BH3)</f>
-        <v>1</v>
+        <v>0.66049382716049387</v>
       </c>
       <c r="BI4">
         <f>IF(BI3&lt;DMAX($A$1:$L$540,$W4,BI$1:BI$2),DMAX($A$1:$L$540,$W4,BI$1:BI$2),BI3)</f>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="BJ4">
         <f>IF(BJ3&lt;DMAX($A$1:$L$540,$W4,BJ$1:BJ$2),DMAX($A$1:$L$540,$W4,BJ$1:BJ$2),BJ3)</f>
-        <v>0.33962264150943394</v>
+        <v>0</v>
       </c>
       <c r="BK4">
         <f>IF(BK3&lt;DMAX($A$1:$L$540,$W4,BK$1:BK$2),DMAX($A$1:$L$540,$W4,BK$1:BK$2),BK3)</f>
-        <v>6.7842605156037995E-3</v>
+        <v>0.33962264150943394</v>
       </c>
       <c r="BL4">
         <f>IF(BL3&lt;DMAX($A$1:$L$540,$W4,BL$1:BL$2),DMAX($A$1:$L$540,$W4,BL$1:BL$2),BL3)</f>
-        <v>8.4210526315789472E-3</v>
+        <v>6.7842605156037995E-3</v>
       </c>
       <c r="BM4">
         <f>IF(BM3&lt;DMAX($A$1:$L$540,$W4,BM$1:BM$2),DMAX($A$1:$L$540,$W4,BM$1:BM$2),BM3)</f>
-        <v>8.2372322899505763E-3</v>
+        <v>8.4210526315789472E-3</v>
       </c>
       <c r="BN4">
         <f>IF(BN3&lt;DMAX($A$1:$L$540,$W4,BN$1:BN$2),DMAX($A$1:$L$540,$W4,BN$1:BN$2),BN3)</f>
-        <v>0</v>
+        <v>8.2372322899505763E-3</v>
       </c>
       <c r="BO4">
         <f>IF(BO3&lt;DMAX($A$1:$L$540,$W4,BO$1:BO$2),DMAX($A$1:$L$540,$W4,BO$1:BO$2),BO3)</f>
@@ -25024,71 +25048,71 @@
       </c>
       <c r="BQ4">
         <f>IF(BQ3&lt;DMAX($A$1:$L$540,$W4,BQ$1:BQ$2),DMAX($A$1:$L$540,$W4,BQ$1:BQ$2),BQ3)</f>
-        <v>0.34693877551020408</v>
+        <v>0</v>
       </c>
       <c r="BR4">
         <f>IF(BR3&lt;DMAX($A$1:$L$540,$W4,BR$1:BR$2),DMAX($A$1:$L$540,$W4,BR$1:BR$2),BR3)</f>
-        <v>0</v>
+        <v>0.34693877551020408</v>
       </c>
       <c r="BS4">
         <f>IF(BS3&lt;DMAX($A$1:$L$540,$W4,BS$1:BS$2),DMAX($A$1:$L$540,$W4,BS$1:BS$2),BS3)</f>
-        <v>0.51327433628318586</v>
+        <v>0</v>
       </c>
       <c r="BT4">
         <f>IF(BT3&lt;DMAX($A$1:$L$540,$W4,BT$1:BT$2),DMAX($A$1:$L$540,$W4,BT$1:BT$2),BT3)</f>
-        <v>1</v>
+        <v>0.51327433628318586</v>
       </c>
       <c r="BU4">
         <f>IF(BU3&lt;DMAX($A$1:$L$540,$W4,BU$1:BU$2),DMAX($A$1:$L$540,$W4,BU$1:BU$2),BU3)</f>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="BV4">
         <f>IF(BV3&lt;DMAX($A$1:$L$540,$W4,BV$1:BV$2),DMAX($A$1:$L$540,$W4,BV$1:BV$2),BV3)</f>
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="BW4">
         <f>IF(BW3&lt;DMAX($A$1:$L$540,$W4,BW$1:BW$2),DMAX($A$1:$L$540,$W4,BW$1:BW$2),BW3)</f>
-        <v>0.65753424657534243</v>
+        <v>1</v>
       </c>
       <c r="BX4">
         <f>IF(BX3&lt;DMAX($A$1:$L$540,$W4,BX$1:BX$2),DMAX($A$1:$L$540,$W4,BX$1:BX$2),BX3)</f>
-        <v>0.44715447154471544</v>
+        <v>0.65753424657534243</v>
       </c>
       <c r="BY4">
         <f>IF(BY3&lt;DMAX($A$1:$L$540,$W4,BY$1:BY$2),DMAX($A$1:$L$540,$W4,BY$1:BY$2),BY3)</f>
-        <v>0.30303030303030304</v>
+        <v>0.44715447154471544</v>
       </c>
       <c r="BZ4">
         <f>IF(BZ3&lt;DMAX($A$1:$L$540,$W4,BZ$1:BZ$2),DMAX($A$1:$L$540,$W4,BZ$1:BZ$2),BZ3)</f>
-        <v>0.38</v>
+        <v>0.30303030303030304</v>
       </c>
       <c r="CA4">
         <f>IF(CA3&lt;DMAX($A$1:$L$540,$W4,CA$1:CA$2),DMAX($A$1:$L$540,$W4,CA$1:CA$2),CA3)</f>
-        <v>0.66666666666666663</v>
+        <v>0.38</v>
       </c>
       <c r="CB4">
         <f>IF(CB3&lt;DMAX($A$1:$L$540,$W4,CB$1:CB$2),DMAX($A$1:$L$540,$W4,CB$1:CB$2),CB3)</f>
-        <v>0</v>
+        <v>0.66666666666666663</v>
       </c>
       <c r="CC4">
         <f>IF(CC3&lt;DMAX($A$1:$L$540,$W4,CC$1:CC$2),DMAX($A$1:$L$540,$W4,CC$1:CC$2),CC3)</f>
-        <v>7.9545454545454544E-2</v>
+        <v>0</v>
       </c>
       <c r="CD4">
         <f>IF(CD3&lt;DMAX($A$1:$L$540,$W4,CD$1:CD$2),DMAX($A$1:$L$540,$W4,CD$1:CD$2),CD3)</f>
-        <v>0.125</v>
+        <v>7.9545454545454544E-2</v>
       </c>
       <c r="CE4">
         <f>IF(CE3&lt;DMAX($A$1:$L$540,$W4,CE$1:CE$2),DMAX($A$1:$L$540,$W4,CE$1:CE$2),CE3)</f>
-        <v>0</v>
+        <v>0.125</v>
       </c>
       <c r="CF4">
         <f>IF(CF3&lt;DMAX($A$1:$L$540,$W4,CF$1:CF$2),DMAX($A$1:$L$540,$W4,CF$1:CF$2),CF3)</f>
-        <v>0.352112676056338</v>
+        <v>0</v>
       </c>
       <c r="CG4">
         <f>IF(CG3&lt;DMAX($A$1:$L$540,$W4,CG$1:CG$2),DMAX($A$1:$L$540,$W4,CG$1:CG$2),CG3)</f>
-        <v>0</v>
+        <v>0.352112676056338</v>
       </c>
       <c r="CH4">
         <f>IF(CH3&lt;DMAX($A$1:$L$540,$W4,CH$1:CH$2),DMAX($A$1:$L$540,$W4,CH$1:CH$2),CH3)</f>
@@ -25098,8 +25122,12 @@
         <f>IF(CI3&lt;DMAX($A$1:$L$540,$W4,CI$1:CI$2),DMAX($A$1:$L$540,$W4,CI$1:CI$2),CI3)</f>
         <v>0</v>
       </c>
-    </row>
-    <row r="5" spans="1:87">
+      <c r="CJ4">
+        <f>IF(CJ3&lt;DMAX($A$1:$L$540,$W4,CJ$1:CJ$2),DMAX($A$1:$L$540,$W4,CJ$1:CJ$2),CJ3)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="5" spans="1:88">
       <c r="A5" t="s">
         <v>458</v>
       </c>
@@ -25153,14 +25181,14 @@
       </c>
       <c r="O5" s="4">
         <f t="shared" si="8"/>
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="P5" t="s">
         <v>892</v>
       </c>
       <c r="Q5" s="8">
         <f t="shared" si="9"/>
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="R5" s="8">
         <f t="shared" si="10"/>
@@ -25179,7 +25207,7 @@
         <v>5</v>
       </c>
       <c r="V5" s="8">
-        <f>COUNTIF($X5:$CI5,"=1")</f>
+        <f>COUNTIF($X5:$CJ5,"=1")</f>
         <v>15</v>
       </c>
       <c r="W5" t="s">
@@ -25243,27 +25271,27 @@
       </c>
       <c r="AL5">
         <f>IF(AL4&lt;DMAX($A$1:$L$540,$W5,AL$1:AL$2),DMAX($A$1:$L$540,$W5,AL$1:AL$2),AL4)</f>
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="AM5">
         <f>IF(AM4&lt;DMAX($A$1:$L$540,$W5,AM$1:AM$2),DMAX($A$1:$L$540,$W5,AM$1:AM$2),AM4)</f>
-        <v>0.68229166666666663</v>
+        <v>1</v>
       </c>
       <c r="AN5">
         <f>IF(AN4&lt;DMAX($A$1:$L$540,$W5,AN$1:AN$2),DMAX($A$1:$L$540,$W5,AN$1:AN$2),AN4)</f>
-        <v>0.52542372881355937</v>
+        <v>0.68229166666666663</v>
       </c>
       <c r="AO5">
         <f>IF(AO4&lt;DMAX($A$1:$L$540,$W5,AO$1:AO$2),DMAX($A$1:$L$540,$W5,AO$1:AO$2),AO4)</f>
-        <v>0.38636363636363635</v>
+        <v>0.52542372881355937</v>
       </c>
       <c r="AP5">
         <f>IF(AP4&lt;DMAX($A$1:$L$540,$W5,AP$1:AP$2),DMAX($A$1:$L$540,$W5,AP$1:AP$2),AP4)</f>
-        <v>0.24848484848484848</v>
+        <v>0.38636363636363635</v>
       </c>
       <c r="AQ5">
         <f>IF(AQ4&lt;DMAX($A$1:$L$540,$W5,AQ$1:AQ$2),DMAX($A$1:$L$540,$W5,AQ$1:AQ$2),AQ4)</f>
-        <v>0</v>
+        <v>0.24848484848484848</v>
       </c>
       <c r="AR5">
         <f>IF(AR4&lt;DMAX($A$1:$L$540,$W5,AR$1:AR$2),DMAX($A$1:$L$540,$W5,AR$1:AR$2),AR4)</f>
@@ -25275,35 +25303,35 @@
       </c>
       <c r="AT5">
         <f>IF(AT4&lt;DMAX($A$1:$L$540,$W5,AT$1:AT$2),DMAX($A$1:$L$540,$W5,AT$1:AT$2),AT4)</f>
-        <v>0.14634146341463414</v>
+        <v>0</v>
       </c>
       <c r="AU5">
         <f>IF(AU4&lt;DMAX($A$1:$L$540,$W5,AU$1:AU$2),DMAX($A$1:$L$540,$W5,AU$1:AU$2),AU4)</f>
-        <v>1</v>
+        <v>0.14634146341463414</v>
       </c>
       <c r="AV5">
         <f>IF(AV4&lt;DMAX($A$1:$L$540,$W5,AV$1:AV$2),DMAX($A$1:$L$540,$W5,AV$1:AV$2),AV4)</f>
-        <v>0.5178571428571429</v>
+        <v>1</v>
       </c>
       <c r="AW5">
         <f>IF(AW4&lt;DMAX($A$1:$L$540,$W5,AW$1:AW$2),DMAX($A$1:$L$540,$W5,AW$1:AW$2),AW4)</f>
-        <v>0.36046511627906974</v>
+        <v>0.5178571428571429</v>
       </c>
       <c r="AX5">
         <f>IF(AX4&lt;DMAX($A$1:$L$540,$W5,AX$1:AX$2),DMAX($A$1:$L$540,$W5,AX$1:AX$2),AX4)</f>
-        <v>0.45652173913043476</v>
+        <v>0.36046511627906974</v>
       </c>
       <c r="AY5">
         <f>IF(AY4&lt;DMAX($A$1:$L$540,$W5,AY$1:AY$2),DMAX($A$1:$L$540,$W5,AY$1:AY$2),AY4)</f>
-        <v>0.43333333333333335</v>
+        <v>0.45652173913043476</v>
       </c>
       <c r="AZ5">
         <f>IF(AZ4&lt;DMAX($A$1:$L$540,$W5,AZ$1:AZ$2),DMAX($A$1:$L$540,$W5,AZ$1:AZ$2),AZ4)</f>
-        <v>0</v>
+        <v>0.43333333333333335</v>
       </c>
       <c r="BA5">
         <f>IF(BA4&lt;DMAX($A$1:$L$540,$W5,BA$1:BA$2),DMAX($A$1:$L$540,$W5,BA$1:BA$2),BA4)</f>
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="BB5">
         <f>IF(BB4&lt;DMAX($A$1:$L$540,$W5,BB$1:BB$2),DMAX($A$1:$L$540,$W5,BB$1:BB$2),BB4)</f>
@@ -25315,15 +25343,15 @@
       </c>
       <c r="BD5">
         <f>IF(BD4&lt;DMAX($A$1:$L$540,$W5,BD$1:BD$2),DMAX($A$1:$L$540,$W5,BD$1:BD$2),BD4)</f>
-        <v>0.36363636363636365</v>
+        <v>1</v>
       </c>
       <c r="BE5">
         <f>IF(BE4&lt;DMAX($A$1:$L$540,$W5,BE$1:BE$2),DMAX($A$1:$L$540,$W5,BE$1:BE$2),BE4)</f>
-        <v>0.47619047619047616</v>
+        <v>0.36363636363636365</v>
       </c>
       <c r="BF5">
         <f>IF(BF4&lt;DMAX($A$1:$L$540,$W5,BF$1:BF$2),DMAX($A$1:$L$540,$W5,BF$1:BF$2),BF4)</f>
-        <v>1</v>
+        <v>0.47619047619047616</v>
       </c>
       <c r="BG5">
         <f>IF(BG4&lt;DMAX($A$1:$L$540,$W5,BG$1:BG$2),DMAX($A$1:$L$540,$W5,BG$1:BG$2),BG4)</f>
@@ -25335,27 +25363,27 @@
       </c>
       <c r="BI5">
         <f>IF(BI4&lt;DMAX($A$1:$L$540,$W5,BI$1:BI$2),DMAX($A$1:$L$540,$W5,BI$1:BI$2),BI4)</f>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="BJ5">
         <f>IF(BJ4&lt;DMAX($A$1:$L$540,$W5,BJ$1:BJ$2),DMAX($A$1:$L$540,$W5,BJ$1:BJ$2),BJ4)</f>
-        <v>0.33962264150943394</v>
+        <v>0</v>
       </c>
       <c r="BK5">
         <f>IF(BK4&lt;DMAX($A$1:$L$540,$W5,BK$1:BK$2),DMAX($A$1:$L$540,$W5,BK$1:BK$2),BK4)</f>
-        <v>6.7842605156037995E-3</v>
+        <v>0.33962264150943394</v>
       </c>
       <c r="BL5">
         <f>IF(BL4&lt;DMAX($A$1:$L$540,$W5,BL$1:BL$2),DMAX($A$1:$L$540,$W5,BL$1:BL$2),BL4)</f>
-        <v>8.4210526315789472E-3</v>
+        <v>6.7842605156037995E-3</v>
       </c>
       <c r="BM5">
         <f>IF(BM4&lt;DMAX($A$1:$L$540,$W5,BM$1:BM$2),DMAX($A$1:$L$540,$W5,BM$1:BM$2),BM4)</f>
-        <v>8.2372322899505763E-3</v>
+        <v>8.4210526315789472E-3</v>
       </c>
       <c r="BN5">
         <f>IF(BN4&lt;DMAX($A$1:$L$540,$W5,BN$1:BN$2),DMAX($A$1:$L$540,$W5,BN$1:BN$2),BN4)</f>
-        <v>1</v>
+        <v>8.2372322899505763E-3</v>
       </c>
       <c r="BO5">
         <f>IF(BO4&lt;DMAX($A$1:$L$540,$W5,BO$1:BO$2),DMAX($A$1:$L$540,$W5,BO$1:BO$2),BO4)</f>
@@ -25363,19 +25391,19 @@
       </c>
       <c r="BP5">
         <f>IF(BP4&lt;DMAX($A$1:$L$540,$W5,BP$1:BP$2),DMAX($A$1:$L$540,$W5,BP$1:BP$2),BP4)</f>
-        <v>0.74603174603174605</v>
+        <v>1</v>
       </c>
       <c r="BQ5">
         <f>IF(BQ4&lt;DMAX($A$1:$L$540,$W5,BQ$1:BQ$2),DMAX($A$1:$L$540,$W5,BQ$1:BQ$2),BQ4)</f>
-        <v>0.34693877551020408</v>
+        <v>0.74603174603174605</v>
       </c>
       <c r="BR5">
         <f>IF(BR4&lt;DMAX($A$1:$L$540,$W5,BR$1:BR$2),DMAX($A$1:$L$540,$W5,BR$1:BR$2),BR4)</f>
-        <v>0.1</v>
+        <v>0.34693877551020408</v>
       </c>
       <c r="BS5">
         <f>IF(BS4&lt;DMAX($A$1:$L$540,$W5,BS$1:BS$2),DMAX($A$1:$L$540,$W5,BS$1:BS$2),BS4)</f>
-        <v>1</v>
+        <v>0.1</v>
       </c>
       <c r="BT5">
         <f>IF(BT4&lt;DMAX($A$1:$L$540,$W5,BT$1:BT$2),DMAX($A$1:$L$540,$W5,BT$1:BT$2),BT4)</f>
@@ -25383,55 +25411,55 @@
       </c>
       <c r="BU5">
         <f>IF(BU4&lt;DMAX($A$1:$L$540,$W5,BU$1:BU$2),DMAX($A$1:$L$540,$W5,BU$1:BU$2),BU4)</f>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="BV5">
         <f>IF(BV4&lt;DMAX($A$1:$L$540,$W5,BV$1:BV$2),DMAX($A$1:$L$540,$W5,BV$1:BV$2),BV4)</f>
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="BW5">
         <f>IF(BW4&lt;DMAX($A$1:$L$540,$W5,BW$1:BW$2),DMAX($A$1:$L$540,$W5,BW$1:BW$2),BW4)</f>
-        <v>0.78082191780821919</v>
+        <v>1</v>
       </c>
       <c r="BX5">
         <f>IF(BX4&lt;DMAX($A$1:$L$540,$W5,BX$1:BX$2),DMAX($A$1:$L$540,$W5,BX$1:BX$2),BX4)</f>
-        <v>0.57723577235772361</v>
+        <v>0.78082191780821919</v>
       </c>
       <c r="BY5">
         <f>IF(BY4&lt;DMAX($A$1:$L$540,$W5,BY$1:BY$2),DMAX($A$1:$L$540,$W5,BY$1:BY$2),BY4)</f>
-        <v>0.66666666666666663</v>
+        <v>0.57723577235772361</v>
       </c>
       <c r="BZ5">
         <f>IF(BZ4&lt;DMAX($A$1:$L$540,$W5,BZ$1:BZ$2),DMAX($A$1:$L$540,$W5,BZ$1:BZ$2),BZ4)</f>
-        <v>0.88</v>
+        <v>0.66666666666666663</v>
       </c>
       <c r="CA5">
         <f>IF(CA4&lt;DMAX($A$1:$L$540,$W5,CA$1:CA$2),DMAX($A$1:$L$540,$W5,CA$1:CA$2),CA4)</f>
-        <v>0.77777777777777779</v>
+        <v>0.88</v>
       </c>
       <c r="CB5">
         <f>IF(CB4&lt;DMAX($A$1:$L$540,$W5,CB$1:CB$2),DMAX($A$1:$L$540,$W5,CB$1:CB$2),CB4)</f>
-        <v>0</v>
+        <v>0.77777777777777779</v>
       </c>
       <c r="CC5">
         <f>IF(CC4&lt;DMAX($A$1:$L$540,$W5,CC$1:CC$2),DMAX($A$1:$L$540,$W5,CC$1:CC$2),CC4)</f>
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="CD5">
         <f>IF(CD4&lt;DMAX($A$1:$L$540,$W5,CD$1:CD$2),DMAX($A$1:$L$540,$W5,CD$1:CD$2),CD4)</f>
-        <v>0.7678571428571429</v>
+        <v>1</v>
       </c>
       <c r="CE5">
         <f>IF(CE4&lt;DMAX($A$1:$L$540,$W5,CE$1:CE$2),DMAX($A$1:$L$540,$W5,CE$1:CE$2),CE4)</f>
-        <v>0</v>
+        <v>0.7678571428571429</v>
       </c>
       <c r="CF5">
         <f>IF(CF4&lt;DMAX($A$1:$L$540,$W5,CF$1:CF$2),DMAX($A$1:$L$540,$W5,CF$1:CF$2),CF4)</f>
-        <v>0.70422535211267601</v>
+        <v>0</v>
       </c>
       <c r="CG5">
         <f>IF(CG4&lt;DMAX($A$1:$L$540,$W5,CG$1:CG$2),DMAX($A$1:$L$540,$W5,CG$1:CG$2),CG4)</f>
-        <v>0</v>
+        <v>0.70422535211267601</v>
       </c>
       <c r="CH5">
         <f>IF(CH4&lt;DMAX($A$1:$L$540,$W5,CH$1:CH$2),DMAX($A$1:$L$540,$W5,CH$1:CH$2),CH4)</f>
@@ -25441,8 +25469,12 @@
         <f>IF(CI4&lt;DMAX($A$1:$L$540,$W5,CI$1:CI$2),DMAX($A$1:$L$540,$W5,CI$1:CI$2),CI4)</f>
         <v>0</v>
       </c>
-    </row>
-    <row r="6" spans="1:87">
+      <c r="CJ5">
+        <f>IF(CJ4&lt;DMAX($A$1:$L$540,$W5,CJ$1:CJ$2),DMAX($A$1:$L$540,$W5,CJ$1:CJ$2),CJ4)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="6" spans="1:88">
       <c r="A6" t="s">
         <v>458</v>
       </c>
@@ -25496,14 +25528,14 @@
       </c>
       <c r="O6" s="4">
         <f t="shared" si="8"/>
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="P6" t="s">
         <v>967</v>
       </c>
       <c r="Q6" s="8">
         <f t="shared" si="9"/>
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="R6" s="8">
         <f t="shared" si="10"/>
@@ -25586,67 +25618,67 @@
       </c>
       <c r="AL6">
         <f>IF(AL5&lt;DMAX($A$1:$L$540,$W6,AL$1:AL$2),DMAX($A$1:$L$540,$W6,AL$1:AL$2),AL5)</f>
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="AM6">
         <f>IF(AM5&lt;DMAX($A$1:$L$540,$W6,AM$1:AM$2),DMAX($A$1:$L$540,$W6,AM$1:AM$2),AM5)</f>
-        <v>0.68229166666666663</v>
+        <v>1</v>
       </c>
       <c r="AN6">
         <f>IF(AN5&lt;DMAX($A$1:$L$540,$W6,AN$1:AN$2),DMAX($A$1:$L$540,$W6,AN$1:AN$2),AN5)</f>
-        <v>1</v>
+        <v>0.68229166666666663</v>
       </c>
       <c r="AO6">
         <f>IF(AO5&lt;DMAX($A$1:$L$540,$W6,AO$1:AO$2),DMAX($A$1:$L$540,$W6,AO$1:AO$2),AO5)</f>
-        <v>0.38636363636363635</v>
+        <v>1</v>
       </c>
       <c r="AP6">
         <f>IF(AP5&lt;DMAX($A$1:$L$540,$W6,AP$1:AP$2),DMAX($A$1:$L$540,$W6,AP$1:AP$2),AP5)</f>
-        <v>0.24848484848484848</v>
+        <v>0.38636363636363635</v>
       </c>
       <c r="AQ6">
         <f>IF(AQ5&lt;DMAX($A$1:$L$540,$W6,AQ$1:AQ$2),DMAX($A$1:$L$540,$W6,AQ$1:AQ$2),AQ5)</f>
-        <v>0.84036144578313254</v>
+        <v>0.24848484848484848</v>
       </c>
       <c r="AR6">
         <f>IF(AR5&lt;DMAX($A$1:$L$540,$W6,AR$1:AR$2),DMAX($A$1:$L$540,$W6,AR$1:AR$2),AR5)</f>
-        <v>0</v>
+        <v>0.84036144578313254</v>
       </c>
       <c r="AS6">
         <f>IF(AS5&lt;DMAX($A$1:$L$540,$W6,AS$1:AS$2),DMAX($A$1:$L$540,$W6,AS$1:AS$2),AS5)</f>
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="AT6">
         <f>IF(AT5&lt;DMAX($A$1:$L$540,$W6,AT$1:AT$2),DMAX($A$1:$L$540,$W6,AT$1:AT$2),AT5)</f>
-        <v>0.17073170731707318</v>
+        <v>1</v>
       </c>
       <c r="AU6">
         <f>IF(AU5&lt;DMAX($A$1:$L$540,$W6,AU$1:AU$2),DMAX($A$1:$L$540,$W6,AU$1:AU$2),AU5)</f>
-        <v>1</v>
+        <v>0.17073170731707318</v>
       </c>
       <c r="AV6">
         <f>IF(AV5&lt;DMAX($A$1:$L$540,$W6,AV$1:AV$2),DMAX($A$1:$L$540,$W6,AV$1:AV$2),AV5)</f>
-        <v>0.5178571428571429</v>
+        <v>1</v>
       </c>
       <c r="AW6">
         <f>IF(AW5&lt;DMAX($A$1:$L$540,$W6,AW$1:AW$2),DMAX($A$1:$L$540,$W6,AW$1:AW$2),AW5)</f>
-        <v>0.81395348837209303</v>
+        <v>0.5178571428571429</v>
       </c>
       <c r="AX6">
         <f>IF(AX5&lt;DMAX($A$1:$L$540,$W6,AX$1:AX$2),DMAX($A$1:$L$540,$W6,AX$1:AX$2),AX5)</f>
-        <v>0.45652173913043476</v>
+        <v>0.81395348837209303</v>
       </c>
       <c r="AY6">
         <f>IF(AY5&lt;DMAX($A$1:$L$540,$W6,AY$1:AY$2),DMAX($A$1:$L$540,$W6,AY$1:AY$2),AY5)</f>
-        <v>0.93333333333333335</v>
+        <v>0.45652173913043476</v>
       </c>
       <c r="AZ6">
         <f>IF(AZ5&lt;DMAX($A$1:$L$540,$W6,AZ$1:AZ$2),DMAX($A$1:$L$540,$W6,AZ$1:AZ$2),AZ5)</f>
-        <v>0</v>
+        <v>0.93333333333333335</v>
       </c>
       <c r="BA6">
         <f>IF(BA5&lt;DMAX($A$1:$L$540,$W6,BA$1:BA$2),DMAX($A$1:$L$540,$W6,BA$1:BA$2),BA5)</f>
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="BB6">
         <f>IF(BB5&lt;DMAX($A$1:$L$540,$W6,BB$1:BB$2),DMAX($A$1:$L$540,$W6,BB$1:BB$2),BB5)</f>
@@ -25658,11 +25690,11 @@
       </c>
       <c r="BD6">
         <f>IF(BD5&lt;DMAX($A$1:$L$540,$W6,BD$1:BD$2),DMAX($A$1:$L$540,$W6,BD$1:BD$2),BD5)</f>
-        <v>0.54545454545454541</v>
+        <v>1</v>
       </c>
       <c r="BE6">
         <f>IF(BE5&lt;DMAX($A$1:$L$540,$W6,BE$1:BE$2),DMAX($A$1:$L$540,$W6,BE$1:BE$2),BE5)</f>
-        <v>1</v>
+        <v>0.54545454545454541</v>
       </c>
       <c r="BF6">
         <f>IF(BF5&lt;DMAX($A$1:$L$540,$W6,BF$1:BF$2),DMAX($A$1:$L$540,$W6,BF$1:BF$2),BF5)</f>
@@ -25678,27 +25710,27 @@
       </c>
       <c r="BI6">
         <f>IF(BI5&lt;DMAX($A$1:$L$540,$W6,BI$1:BI$2),DMAX($A$1:$L$540,$W6,BI$1:BI$2),BI5)</f>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="BJ6">
         <f>IF(BJ5&lt;DMAX($A$1:$L$540,$W6,BJ$1:BJ$2),DMAX($A$1:$L$540,$W6,BJ$1:BJ$2),BJ5)</f>
-        <v>0.33962264150943394</v>
+        <v>0</v>
       </c>
       <c r="BK6">
         <f>IF(BK5&lt;DMAX($A$1:$L$540,$W6,BK$1:BK$2),DMAX($A$1:$L$540,$W6,BK$1:BK$2),BK5)</f>
-        <v>6.7842605156037995E-3</v>
+        <v>0.33962264150943394</v>
       </c>
       <c r="BL6">
         <f>IF(BL5&lt;DMAX($A$1:$L$540,$W6,BL$1:BL$2),DMAX($A$1:$L$540,$W6,BL$1:BL$2),BL5)</f>
-        <v>8.4210526315789472E-3</v>
+        <v>6.7842605156037995E-3</v>
       </c>
       <c r="BM6">
         <f>IF(BM5&lt;DMAX($A$1:$L$540,$W6,BM$1:BM$2),DMAX($A$1:$L$540,$W6,BM$1:BM$2),BM5)</f>
-        <v>8.2372322899505763E-3</v>
+        <v>8.4210526315789472E-3</v>
       </c>
       <c r="BN6">
         <f>IF(BN5&lt;DMAX($A$1:$L$540,$W6,BN$1:BN$2),DMAX($A$1:$L$540,$W6,BN$1:BN$2),BN5)</f>
-        <v>1</v>
+        <v>8.2372322899505763E-3</v>
       </c>
       <c r="BO6">
         <f>IF(BO5&lt;DMAX($A$1:$L$540,$W6,BO$1:BO$2),DMAX($A$1:$L$540,$W6,BO$1:BO$2),BO5)</f>
@@ -25706,19 +25738,19 @@
       </c>
       <c r="BP6">
         <f>IF(BP5&lt;DMAX($A$1:$L$540,$W6,BP$1:BP$2),DMAX($A$1:$L$540,$W6,BP$1:BP$2),BP5)</f>
-        <v>0.74603174603174605</v>
+        <v>1</v>
       </c>
       <c r="BQ6">
         <f>IF(BQ5&lt;DMAX($A$1:$L$540,$W6,BQ$1:BQ$2),DMAX($A$1:$L$540,$W6,BQ$1:BQ$2),BQ5)</f>
-        <v>0.34693877551020408</v>
+        <v>0.74603174603174605</v>
       </c>
       <c r="BR6">
         <f>IF(BR5&lt;DMAX($A$1:$L$540,$W6,BR$1:BR$2),DMAX($A$1:$L$540,$W6,BR$1:BR$2),BR5)</f>
-        <v>0.6</v>
+        <v>0.34693877551020408</v>
       </c>
       <c r="BS6">
         <f>IF(BS5&lt;DMAX($A$1:$L$540,$W6,BS$1:BS$2),DMAX($A$1:$L$540,$W6,BS$1:BS$2),BS5)</f>
-        <v>1</v>
+        <v>0.6</v>
       </c>
       <c r="BT6">
         <f>IF(BT5&lt;DMAX($A$1:$L$540,$W6,BT$1:BT$2),DMAX($A$1:$L$540,$W6,BT$1:BT$2),BT5)</f>
@@ -25726,11 +25758,11 @@
       </c>
       <c r="BU6">
         <f>IF(BU5&lt;DMAX($A$1:$L$540,$W6,BU$1:BU$2),DMAX($A$1:$L$540,$W6,BU$1:BU$2),BU5)</f>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="BV6">
         <f>IF(BV5&lt;DMAX($A$1:$L$540,$W6,BV$1:BV$2),DMAX($A$1:$L$540,$W6,BV$1:BV$2),BV5)</f>
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="BW6">
         <f>IF(BW5&lt;DMAX($A$1:$L$540,$W6,BW$1:BW$2),DMAX($A$1:$L$540,$W6,BW$1:BW$2),BW5)</f>
@@ -25742,11 +25774,11 @@
       </c>
       <c r="BY6">
         <f>IF(BY5&lt;DMAX($A$1:$L$540,$W6,BY$1:BY$2),DMAX($A$1:$L$540,$W6,BY$1:BY$2),BY5)</f>
-        <v>0.66666666666666663</v>
+        <v>1</v>
       </c>
       <c r="BZ6">
         <f>IF(BZ5&lt;DMAX($A$1:$L$540,$W6,BZ$1:BZ$2),DMAX($A$1:$L$540,$W6,BZ$1:BZ$2),BZ5)</f>
-        <v>1</v>
+        <v>0.66666666666666663</v>
       </c>
       <c r="CA6">
         <f>IF(CA5&lt;DMAX($A$1:$L$540,$W6,CA$1:CA$2),DMAX($A$1:$L$540,$W6,CA$1:CA$2),CA5)</f>
@@ -25754,11 +25786,11 @@
       </c>
       <c r="CB6">
         <f>IF(CB5&lt;DMAX($A$1:$L$540,$W6,CB$1:CB$2),DMAX($A$1:$L$540,$W6,CB$1:CB$2),CB5)</f>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="CC6">
         <f>IF(CC5&lt;DMAX($A$1:$L$540,$W6,CC$1:CC$2),DMAX($A$1:$L$540,$W6,CC$1:CC$2),CC5)</f>
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="CD6">
         <f>IF(CD5&lt;DMAX($A$1:$L$540,$W6,CD$1:CD$2),DMAX($A$1:$L$540,$W6,CD$1:CD$2),CD5)</f>
@@ -25766,26 +25798,30 @@
       </c>
       <c r="CE6">
         <f>IF(CE5&lt;DMAX($A$1:$L$540,$W6,CE$1:CE$2),DMAX($A$1:$L$540,$W6,CE$1:CE$2),CE5)</f>
-        <v>0.42857142857142855</v>
+        <v>1</v>
       </c>
       <c r="CF6">
         <f>IF(CF5&lt;DMAX($A$1:$L$540,$W6,CF$1:CF$2),DMAX($A$1:$L$540,$W6,CF$1:CF$2),CF5)</f>
-        <v>1</v>
+        <v>0.42857142857142855</v>
       </c>
       <c r="CG6">
         <f>IF(CG5&lt;DMAX($A$1:$L$540,$W6,CG$1:CG$2),DMAX($A$1:$L$540,$W6,CG$1:CG$2),CG5)</f>
-        <v>0.74193548387096775</v>
+        <v>1</v>
       </c>
       <c r="CH6">
         <f>IF(CH5&lt;DMAX($A$1:$L$540,$W6,CH$1:CH$2),DMAX($A$1:$L$540,$W6,CH$1:CH$2),CH5)</f>
-        <v>0</v>
+        <v>0.74193548387096775</v>
       </c>
       <c r="CI6">
         <f>IF(CI5&lt;DMAX($A$1:$L$540,$W6,CI$1:CI$2),DMAX($A$1:$L$540,$W6,CI$1:CI$2),CI5)</f>
         <v>0</v>
       </c>
-    </row>
-    <row r="7" spans="1:87">
+      <c r="CJ6">
+        <f>IF(CJ5&lt;DMAX($A$1:$L$540,$W6,CJ$1:CJ$2),DMAX($A$1:$L$540,$W6,CJ$1:CJ$2),CJ5)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="7" spans="1:88">
       <c r="A7" t="s">
         <v>458</v>
       </c>
@@ -25832,11 +25868,11 @@
       <c r="M7" s="4"/>
       <c r="N7" s="4">
         <f t="shared" si="7"/>
-        <v>0.96875</v>
+        <v>0.984375</v>
       </c>
       <c r="O7" s="4">
         <f t="shared" si="8"/>
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="P7" s="7" t="s">
         <v>893</v>
@@ -25863,7 +25899,7 @@
       </c>
       <c r="V7" s="8">
         <f t="shared" si="14"/>
-        <v>60</v>
+        <v>61</v>
       </c>
       <c r="W7" s="7" t="s">
         <v>893</v>
@@ -25950,19 +25986,19 @@
       </c>
       <c r="AR7">
         <f>IF(AR6&lt;DMAX($A$1:$L$540,$W7,AR$1:AR$2),DMAX($A$1:$L$540,$W7,AR$1:AR$2),AR6)</f>
-        <v>0.99224806201550386</v>
+        <v>1</v>
       </c>
       <c r="AS7">
         <f>IF(AS6&lt;DMAX($A$1:$L$540,$W7,AS$1:AS$2),DMAX($A$1:$L$540,$W7,AS$1:AS$2),AS6)</f>
-        <v>1</v>
+        <v>0.99224806201550386</v>
       </c>
       <c r="AT7">
         <f>IF(AT6&lt;DMAX($A$1:$L$540,$W7,AT$1:AT$2),DMAX($A$1:$L$540,$W7,AT$1:AT$2),AT6)</f>
-        <v>0.26829268292682928</v>
+        <v>1</v>
       </c>
       <c r="AU7">
         <f>IF(AU6&lt;DMAX($A$1:$L$540,$W7,AU$1:AU$2),DMAX($A$1:$L$540,$W7,AU$1:AU$2),AU6)</f>
-        <v>1</v>
+        <v>0.26829268292682928</v>
       </c>
       <c r="AV7">
         <f>IF(AV6&lt;DMAX($A$1:$L$540,$W7,AV$1:AV$2),DMAX($A$1:$L$540,$W7,AV$1:AV$2),AV6)</f>
@@ -26018,11 +26054,11 @@
       </c>
       <c r="BI7">
         <f>IF(BI6&lt;DMAX($A$1:$L$540,$W7,BI$1:BI$2),DMAX($A$1:$L$540,$W7,BI$1:BI$2),BI6)</f>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="BJ7">
         <f>IF(BJ6&lt;DMAX($A$1:$L$540,$W7,BJ$1:BJ$2),DMAX($A$1:$L$540,$W7,BJ$1:BJ$2),BJ6)</f>
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="BK7">
         <f>IF(BK6&lt;DMAX($A$1:$L$540,$W7,BK$1:BK$2),DMAX($A$1:$L$540,$W7,BK$1:BK$2),BK6)</f>
@@ -26046,11 +26082,11 @@
       </c>
       <c r="BP7">
         <f>IF(BP6&lt;DMAX($A$1:$L$540,$W7,BP$1:BP$2),DMAX($A$1:$L$540,$W7,BP$1:BP$2),BP6)</f>
-        <v>0.74603174603174605</v>
+        <v>1</v>
       </c>
       <c r="BQ7">
         <f>IF(BQ6&lt;DMAX($A$1:$L$540,$W7,BQ$1:BQ$2),DMAX($A$1:$L$540,$W7,BQ$1:BQ$2),BQ6)</f>
-        <v>1</v>
+        <v>0.74603174603174605</v>
       </c>
       <c r="BR7">
         <f>IF(BR6&lt;DMAX($A$1:$L$540,$W7,BR$1:BR$2),DMAX($A$1:$L$540,$W7,BR$1:BR$2),BR6)</f>
@@ -26124,8 +26160,12 @@
         <f>IF(CI6&lt;DMAX($A$1:$L$540,$W7,CI$1:CI$2),DMAX($A$1:$L$540,$W7,CI$1:CI$2),CI6)</f>
         <v>1</v>
       </c>
-    </row>
-    <row r="8" spans="1:87">
+      <c r="CJ7">
+        <f>IF(CJ6&lt;DMAX($A$1:$L$540,$W7,CJ$1:CJ$2),DMAX($A$1:$L$540,$W7,CJ$1:CJ$2),CJ6)</f>
+        <v>1</v>
+      </c>
+    </row>
+    <row r="8" spans="1:88">
       <c r="A8" t="s">
         <v>458</v>
       </c>
@@ -26172,7 +26212,7 @@
       <c r="M8" s="4"/>
       <c r="N8" s="4">
         <f>SUM(T8:V8)/64</f>
-        <v>0.984375</v>
+        <v>1</v>
       </c>
       <c r="O8" s="4"/>
       <c r="P8" s="4" t="s">
@@ -26200,7 +26240,7 @@
       </c>
       <c r="V8" s="8">
         <f t="shared" si="14"/>
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="W8" s="7" t="s">
         <v>968</v>
@@ -26355,11 +26395,11 @@
       </c>
       <c r="BI8">
         <f>IF(BI7&lt;DMAX($A$1:$L$540,$W8,BI$1:BI$2),DMAX($A$1:$L$540,$W8,BI$1:BI$2),BI7)</f>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="BJ8">
         <f>IF(BJ7&lt;DMAX($A$1:$L$540,$W8,BJ$1:BJ$2),DMAX($A$1:$L$540,$W8,BJ$1:BJ$2),BJ7)</f>
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="BK8">
         <f>IF(BK7&lt;DMAX($A$1:$L$540,$W8,BK$1:BK$2),DMAX($A$1:$L$540,$W8,BK$1:BK$2),BK7)</f>
@@ -26383,11 +26423,11 @@
       </c>
       <c r="BP8">
         <f>IF(BP7&lt;DMAX($A$1:$L$540,$W8,BP$1:BP$2),DMAX($A$1:$L$540,$W8,BP$1:BP$2),BP7)</f>
-        <v>0.74603174603174605</v>
+        <v>1</v>
       </c>
       <c r="BQ8">
         <f>IF(BQ7&lt;DMAX($A$1:$L$540,$W8,BQ$1:BQ$2),DMAX($A$1:$L$540,$W8,BQ$1:BQ$2),BQ7)</f>
-        <v>1</v>
+        <v>0.74603174603174605</v>
       </c>
       <c r="BR8">
         <f>IF(BR7&lt;DMAX($A$1:$L$540,$W8,BR$1:BR$2),DMAX($A$1:$L$540,$W8,BR$1:BR$2),BR7)</f>
@@ -26461,8 +26501,12 @@
         <f>IF(CI7&lt;DMAX($A$1:$L$540,$W8,CI$1:CI$2),DMAX($A$1:$L$540,$W8,CI$1:CI$2),CI7)</f>
         <v>1</v>
       </c>
-    </row>
-    <row r="9" spans="1:87">
+      <c r="CJ8">
+        <f>IF(CJ7&lt;DMAX($A$1:$L$540,$W8,CJ$1:CJ$2),DMAX($A$1:$L$540,$W8,CJ$1:CJ$2),CJ7)</f>
+        <v>1</v>
+      </c>
+    </row>
+    <row r="9" spans="1:88">
       <c r="A9" t="s">
         <v>458</v>
       </c>
@@ -26516,7 +26560,7 @@
       <c r="T9" s="4"/>
       <c r="U9" s="4"/>
     </row>
-    <row r="10" spans="1:87">
+    <row r="10" spans="1:88">
       <c r="A10" t="s">
         <v>458</v>
       </c>
@@ -26570,7 +26614,7 @@
       <c r="T10" s="4"/>
       <c r="U10" s="4"/>
     </row>
-    <row r="11" spans="1:87">
+    <row r="11" spans="1:88">
       <c r="A11" t="s">
         <v>458</v>
       </c>
@@ -26624,7 +26668,7 @@
       <c r="T11" s="4"/>
       <c r="U11" s="4"/>
     </row>
-    <row r="12" spans="1:87">
+    <row r="12" spans="1:88">
       <c r="A12" t="s">
         <v>458</v>
       </c>
@@ -26678,7 +26722,7 @@
       <c r="T12" s="4"/>
       <c r="U12" s="4"/>
     </row>
-    <row r="13" spans="1:87">
+    <row r="13" spans="1:88">
       <c r="A13" t="s">
         <v>458</v>
       </c>
@@ -26732,7 +26776,7 @@
       <c r="T13" s="4"/>
       <c r="U13" s="4"/>
     </row>
-    <row r="14" spans="1:87">
+    <row r="14" spans="1:88">
       <c r="A14" t="s">
         <v>458</v>
       </c>
@@ -26786,7 +26830,7 @@
       <c r="T14" s="4"/>
       <c r="U14" s="4"/>
     </row>
-    <row r="15" spans="1:87">
+    <row r="15" spans="1:88">
       <c r="A15" t="s">
         <v>458</v>
       </c>
@@ -26840,7 +26884,7 @@
       <c r="T15" s="4"/>
       <c r="U15" s="4"/>
     </row>
-    <row r="16" spans="1:87">
+    <row r="16" spans="1:88">
       <c r="A16" t="s">
         <v>458</v>
       </c>
@@ -59010,10 +59054,8 @@
       <c r="J14" s="2">
         <v>5</v>
       </c>
-      <c r="N14" s="3" t="s">
-        <v>901</v>
-      </c>
-      <c r="O14" s="3"/>
+      <c r="N14" s="9"/>
+      <c r="O14" s="9"/>
     </row>
     <row r="15" spans="1:15">
       <c r="A15" s="2"/>
@@ -59133,7 +59175,7 @@
         <v>441</v>
       </c>
       <c r="N18" t="s">
-        <v>904</v>
+        <v>970</v>
       </c>
     </row>
     <row r="19" spans="1:14">
@@ -59159,7 +59201,7 @@
       <c r="H19" s="2"/>
       <c r="I19" s="2"/>
       <c r="N19" t="s">
-        <v>916</v>
+        <v>904</v>
       </c>
     </row>
     <row r="20" spans="1:14">
@@ -59185,7 +59227,7 @@
       <c r="H20" s="2"/>
       <c r="I20" s="2"/>
       <c r="N20" t="s">
-        <v>917</v>
+        <v>916</v>
       </c>
     </row>
     <row r="21" spans="1:14">
@@ -59211,7 +59253,7 @@
       <c r="H21" s="2"/>
       <c r="I21" s="2"/>
       <c r="N21" t="s">
-        <v>918</v>
+        <v>917</v>
       </c>
     </row>
     <row r="22" spans="1:14">
@@ -59239,7 +59281,7 @@
       <c r="H22" s="2"/>
       <c r="I22" s="2"/>
       <c r="N22" t="s">
-        <v>919</v>
+        <v>918</v>
       </c>
     </row>
     <row r="23" spans="1:14">
@@ -59277,7 +59319,7 @@
         <v>441</v>
       </c>
       <c r="N23" t="s">
-        <v>920</v>
+        <v>919</v>
       </c>
     </row>
     <row r="24" spans="1:14">
@@ -59313,7 +59355,7 @@
         <v>441</v>
       </c>
       <c r="N24" t="s">
-        <v>921</v>
+        <v>920</v>
       </c>
     </row>
     <row r="25" spans="1:14">
@@ -59349,7 +59391,7 @@
         <v>441</v>
       </c>
       <c r="N25" t="s">
-        <v>922</v>
+        <v>921</v>
       </c>
     </row>
     <row r="26" spans="1:14">
@@ -59385,7 +59427,7 @@
         <v>441</v>
       </c>
       <c r="N26" t="s">
-        <v>923</v>
+        <v>922</v>
       </c>
     </row>
     <row r="27" spans="1:14">
@@ -59411,7 +59453,7 @@
       <c r="H27" s="2"/>
       <c r="I27" s="2"/>
       <c r="N27" t="s">
-        <v>924</v>
+        <v>923</v>
       </c>
     </row>
     <row r="28" spans="1:14">
@@ -59449,7 +59491,7 @@
         <v>441</v>
       </c>
       <c r="N28" t="s">
-        <v>925</v>
+        <v>924</v>
       </c>
     </row>
     <row r="29" spans="1:14">
@@ -59485,7 +59527,7 @@
         <v>441</v>
       </c>
       <c r="N29" t="s">
-        <v>926</v>
+        <v>925</v>
       </c>
     </row>
     <row r="30" spans="1:14">
@@ -59521,7 +59563,7 @@
         <v>441</v>
       </c>
       <c r="N30" t="s">
-        <v>927</v>
+        <v>926</v>
       </c>
     </row>
     <row r="31" spans="1:14">
@@ -59557,7 +59599,7 @@
         <v>441</v>
       </c>
       <c r="N31" t="s">
-        <v>928</v>
+        <v>927</v>
       </c>
     </row>
     <row r="32" spans="1:14">
@@ -59583,7 +59625,7 @@
       <c r="H32" s="2"/>
       <c r="I32" s="2"/>
       <c r="N32" t="s">
-        <v>929</v>
+        <v>928</v>
       </c>
     </row>
     <row r="33" spans="1:14">
@@ -59621,7 +59663,7 @@
         <v>441</v>
       </c>
       <c r="N33" t="s">
-        <v>930</v>
+        <v>929</v>
       </c>
     </row>
     <row r="34" spans="1:14">
@@ -59649,7 +59691,7 @@
       <c r="H34" s="2"/>
       <c r="I34" s="2"/>
       <c r="N34" t="s">
-        <v>931</v>
+        <v>930</v>
       </c>
     </row>
     <row r="35" spans="1:14">
@@ -59682,7 +59724,7 @@
         <v>9</v>
       </c>
       <c r="N35" t="s">
-        <v>932</v>
+        <v>931</v>
       </c>
     </row>
     <row r="36" spans="1:14">
@@ -59715,7 +59757,7 @@
         <v>10</v>
       </c>
       <c r="N36" t="s">
-        <v>933</v>
+        <v>932</v>
       </c>
     </row>
     <row r="37" spans="1:14">
@@ -59741,7 +59783,7 @@
       <c r="H37" s="2"/>
       <c r="I37" s="2"/>
       <c r="N37" t="s">
-        <v>934</v>
+        <v>933</v>
       </c>
     </row>
     <row r="38" spans="1:14">
@@ -59767,7 +59809,7 @@
       <c r="H38" s="2"/>
       <c r="I38" s="2"/>
       <c r="N38" t="s">
-        <v>935</v>
+        <v>934</v>
       </c>
     </row>
     <row r="39" spans="1:14">
@@ -59793,7 +59835,7 @@
       <c r="H39" s="2"/>
       <c r="I39" s="2"/>
       <c r="N39" t="s">
-        <v>936</v>
+        <v>935</v>
       </c>
     </row>
     <row r="40" spans="1:14">
@@ -59826,7 +59868,7 @@
         <v>10</v>
       </c>
       <c r="N40" t="s">
-        <v>937</v>
+        <v>936</v>
       </c>
     </row>
     <row r="41" spans="1:14">
@@ -59859,7 +59901,7 @@
         <v>10</v>
       </c>
       <c r="N41" t="s">
-        <v>938</v>
+        <v>937</v>
       </c>
     </row>
     <row r="42" spans="1:14">
@@ -59891,9 +59933,7 @@
       <c r="J42" s="2">
         <v>2</v>
       </c>
-      <c r="N42" t="s">
-        <v>939</v>
-      </c>
+      <c r="N42" s="9"/>
     </row>
     <row r="43" spans="1:14">
       <c r="A43" s="2"/>
@@ -59925,7 +59965,7 @@
         <v>3</v>
       </c>
       <c r="N43" t="s">
-        <v>940</v>
+        <v>939</v>
       </c>
     </row>
     <row r="44" spans="1:14">
@@ -59961,7 +60001,7 @@
         <v>441</v>
       </c>
       <c r="N44" t="s">
-        <v>941</v>
+        <v>940</v>
       </c>
     </row>
     <row r="45" spans="1:14">
@@ -59997,7 +60037,7 @@
         <v>443</v>
       </c>
       <c r="N45" t="s">
-        <v>942</v>
+        <v>971</v>
       </c>
     </row>
     <row r="46" spans="1:14">
@@ -60033,7 +60073,7 @@
         <v>441</v>
       </c>
       <c r="N46" t="s">
-        <v>943</v>
+        <v>941</v>
       </c>
     </row>
     <row r="47" spans="1:14">
@@ -60069,7 +60109,7 @@
         <v>445</v>
       </c>
       <c r="N47" t="s">
-        <v>944</v>
+        <v>942</v>
       </c>
     </row>
     <row r="48" spans="1:14">
@@ -60105,7 +60145,7 @@
         <v>441</v>
       </c>
       <c r="N48" t="s">
-        <v>945</v>
+        <v>943</v>
       </c>
     </row>
     <row r="49" spans="1:14">
@@ -60138,7 +60178,7 @@
         <v>4</v>
       </c>
       <c r="N49" t="s">
-        <v>946</v>
+        <v>944</v>
       </c>
     </row>
     <row r="50" spans="1:14">
@@ -60172,9 +60212,7 @@
       <c r="J50" s="2">
         <v>4</v>
       </c>
-      <c r="N50" t="s">
-        <v>947</v>
-      </c>
+      <c r="N50" s="9"/>
     </row>
     <row r="51" spans="1:14">
       <c r="A51" s="2"/>
@@ -60205,9 +60243,7 @@
       <c r="J51" s="2">
         <v>6</v>
       </c>
-      <c r="N51" t="s">
-        <v>948</v>
-      </c>
+      <c r="N51" s="9"/>
     </row>
     <row r="52" spans="1:14">
       <c r="A52" s="2" t="s">
@@ -60234,7 +60270,7 @@
       <c r="H52" s="2"/>
       <c r="I52" s="2"/>
       <c r="N52" t="s">
-        <v>949</v>
+        <v>947</v>
       </c>
     </row>
     <row r="53" spans="1:14">
@@ -60270,7 +60306,7 @@
         <v>441</v>
       </c>
       <c r="N53" t="s">
-        <v>950</v>
+        <v>948</v>
       </c>
     </row>
     <row r="54" spans="1:14">
@@ -60298,7 +60334,7 @@
       <c r="H54" s="2"/>
       <c r="I54" s="2"/>
       <c r="N54" t="s">
-        <v>951</v>
+        <v>949</v>
       </c>
     </row>
     <row r="55" spans="1:14">
@@ -60332,9 +60368,7 @@
       <c r="J55" s="2">
         <v>2</v>
       </c>
-      <c r="N55" t="s">
-        <v>952</v>
-      </c>
+      <c r="N55" s="9"/>
     </row>
     <row r="56" spans="1:14">
       <c r="A56" s="2" t="s">
@@ -60371,7 +60405,7 @@
         <v>60</v>
       </c>
       <c r="N56" t="s">
-        <v>953</v>
+        <v>951</v>
       </c>
     </row>
     <row r="57" spans="1:14">
@@ -60405,9 +60439,7 @@
       <c r="J57" s="2">
         <v>7</v>
       </c>
-      <c r="N57" t="s">
-        <v>954</v>
-      </c>
+      <c r="N57" s="9"/>
     </row>
     <row r="58" spans="1:14">
       <c r="A58" s="2"/>
@@ -60439,7 +60471,7 @@
         <v>8</v>
       </c>
       <c r="N58" t="s">
-        <v>955</v>
+        <v>953</v>
       </c>
     </row>
     <row r="59" spans="1:14">
@@ -60472,7 +60504,7 @@
         <v>4</v>
       </c>
       <c r="N59" t="s">
-        <v>956</v>
+        <v>954</v>
       </c>
     </row>
     <row r="60" spans="1:14">
@@ -60504,9 +60536,7 @@
       <c r="J60" s="2">
         <v>5</v>
       </c>
-      <c r="N60" t="s">
-        <v>957</v>
-      </c>
+      <c r="N60" s="9"/>
     </row>
     <row r="61" spans="1:14">
       <c r="A61" s="2"/>
@@ -60538,7 +60568,7 @@
         <v>20</v>
       </c>
       <c r="N61" t="s">
-        <v>958</v>
+        <v>956</v>
       </c>
     </row>
     <row r="62" spans="1:14">
@@ -60571,7 +60601,7 @@
         <v>8</v>
       </c>
       <c r="N62" t="s">
-        <v>959</v>
+        <v>957</v>
       </c>
     </row>
     <row r="63" spans="1:14">
@@ -60597,7 +60627,7 @@
       <c r="H63" s="2"/>
       <c r="I63" s="2"/>
       <c r="N63" t="s">
-        <v>960</v>
+        <v>958</v>
       </c>
     </row>
     <row r="64" spans="1:14">
@@ -60623,7 +60653,7 @@
       <c r="H64" s="2"/>
       <c r="I64" s="2"/>
       <c r="N64" t="s">
-        <v>961</v>
+        <v>959</v>
       </c>
     </row>
     <row r="65" spans="1:14">
@@ -60649,7 +60679,7 @@
       <c r="H65" s="2"/>
       <c r="I65" s="2"/>
       <c r="N65" t="s">
-        <v>962</v>
+        <v>960</v>
       </c>
     </row>
     <row r="66" spans="1:14">
@@ -60684,7 +60714,7 @@
         <v>6</v>
       </c>
       <c r="N66" t="s">
-        <v>963</v>
+        <v>961</v>
       </c>
     </row>
     <row r="67" spans="1:14">
@@ -60720,7 +60750,7 @@
         <v>441</v>
       </c>
       <c r="N67" t="s">
-        <v>964</v>
+        <v>962</v>
       </c>
     </row>
     <row r="68" spans="1:14">
@@ -60755,6 +60785,9 @@
       <c r="K68" t="s">
         <v>441</v>
       </c>
+      <c r="N68" t="s">
+        <v>963</v>
+      </c>
     </row>
     <row r="69" spans="1:14">
       <c r="A69" s="2"/>
@@ -60785,6 +60818,7 @@
       <c r="J69" s="2">
         <v>24</v>
       </c>
+      <c r="N69" s="9"/>
     </row>
     <row r="70" spans="1:14">
       <c r="A70" s="2"/>
@@ -64416,6 +64450,9 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="A1:G545"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0"/>
+  <cols>
+    <col min="1" max="1" width="25.33203125" bestFit="1" customWidth="1"/>
+  </cols>
   <sheetData>
     <row r="1" spans="1:7">
       <c r="A1" t="s">

</xml_diff>